<commit_message>
seperate topic lists and more pandas git ex files
</commit_message>
<xml_diff>
--- a/p/py-25/py-core/topic-list_py.xlsx
+++ b/p/py-25/py-core/topic-list_py.xlsx
@@ -2490,7 +2490,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2520,11 +2520,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2971,16 +2969,16 @@
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:8">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="21"/>
     </row>
     <row r="16" spans="3:3">
       <c r="C16" s="1" t="s">
@@ -3003,12 +3001,12 @@
       </c>
     </row>
     <row r="21" spans="4:4">
-      <c r="D21" s="17" t="s">
+      <c r="D21" s="9" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="22" spans="4:5">
-      <c r="D22" s="17"/>
+      <c r="D22" s="9"/>
       <c r="E22" s="1" t="s">
         <v>23</v>
       </c>
@@ -3075,17 +3073,17 @@
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19" t="s">
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" s="19" t="s">
+      <c r="A34" s="17" t="s">
         <v>41</v>
       </c>
       <c r="D34" s="1" t="s">
@@ -3093,7 +3091,7 @@
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="17" t="s">
         <v>43</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -3101,7 +3099,7 @@
       </c>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" s="19"/>
+      <c r="A36" s="17"/>
     </row>
     <row r="37" spans="3:3">
       <c r="C37" s="1" t="s">
@@ -3109,7 +3107,7 @@
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="19" t="s">
+      <c r="A38" s="17" t="s">
         <v>46</v>
       </c>
       <c r="B38" s="1" t="s">
@@ -3135,9 +3133,9 @@
       </c>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" s="20"/>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="18"/>
+      <c r="C43" s="18"/>
       <c r="D43" s="1" t="s">
         <v>52</v>
       </c>
@@ -3189,59 +3187,59 @@
       </c>
     </row>
     <row r="53" spans="3:5">
-      <c r="C53" s="20"/>
-      <c r="D53" s="20"/>
-      <c r="E53" s="20"/>
+      <c r="C53" s="18"/>
+      <c r="D53" s="18"/>
+      <c r="E53" s="18"/>
     </row>
     <row r="54" spans="3:5">
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="20"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="18"/>
     </row>
     <row r="55" spans="3:5">
-      <c r="C55" s="20"/>
-      <c r="D55" s="20"/>
-      <c r="E55" s="20"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="18"/>
     </row>
     <row r="56" spans="3:5">
-      <c r="C56" s="20"/>
-      <c r="D56" s="20"/>
-      <c r="E56" s="20"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
     </row>
     <row r="57" spans="3:5">
-      <c r="C57" s="20"/>
-      <c r="D57" s="20"/>
-      <c r="E57" s="20"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
     </row>
     <row r="58" spans="3:5">
-      <c r="C58" s="20"/>
-      <c r="D58" s="20"/>
-      <c r="E58" s="20"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="18"/>
     </row>
     <row r="59" spans="3:5">
-      <c r="C59" s="20"/>
-      <c r="D59" s="20"/>
-      <c r="E59" s="20"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
     </row>
     <row r="60" spans="3:5">
-      <c r="C60" s="20"/>
-      <c r="D60" s="20"/>
-      <c r="E60" s="20"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
     </row>
     <row r="61" spans="3:5">
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
-      <c r="E61" s="20"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
     </row>
     <row r="62" spans="3:5">
-      <c r="C62" s="20"/>
-      <c r="D62" s="20"/>
-      <c r="E62" s="20"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="18"/>
     </row>
     <row r="63" spans="3:5">
-      <c r="C63" s="20"/>
-      <c r="D63" s="20"/>
-      <c r="E63" s="20"/>
+      <c r="C63" s="18"/>
+      <c r="D63" s="18"/>
+      <c r="E63" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3666,211 +3664,211 @@
       </c>
     </row>
     <row r="6" spans="3:3">
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="7" spans="3:3">
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="9" spans="3:3">
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="19" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="11" spans="3:5">
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
     </row>
     <row r="12" spans="3:5">
-      <c r="C12" s="17"/>
-      <c r="D12" s="22" t="s">
+      <c r="C12" s="9"/>
+      <c r="D12" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="17"/>
+      <c r="E12" s="9"/>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17" t="s">
+      <c r="C13" s="9"/>
+      <c r="D13" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="E13" s="17"/>
+      <c r="E13" s="9"/>
     </row>
     <row r="14" spans="3:5">
-      <c r="C14" s="17"/>
-      <c r="D14" s="17" t="s">
+      <c r="C14" s="9"/>
+      <c r="D14" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="E14" s="17"/>
+      <c r="E14" s="9"/>
     </row>
     <row r="15" spans="3:5">
-      <c r="C15" s="17"/>
-      <c r="D15" s="17" t="s">
+      <c r="C15" s="9"/>
+      <c r="D15" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="E15" s="17"/>
+      <c r="E15" s="9"/>
     </row>
     <row r="16" spans="3:5">
-      <c r="C16" s="17"/>
-      <c r="D16" s="17" t="s">
+      <c r="C16" s="9"/>
+      <c r="D16" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="17"/>
+      <c r="E16" s="9"/>
     </row>
     <row r="17" spans="3:5">
-      <c r="C17" s="17"/>
-      <c r="D17" s="17" t="s">
+      <c r="C17" s="9"/>
+      <c r="D17" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="E17" s="17"/>
+      <c r="E17" s="9"/>
     </row>
     <row r="18" spans="3:5">
-      <c r="C18" s="17"/>
-      <c r="D18" s="17" t="s">
+      <c r="C18" s="9"/>
+      <c r="D18" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="E18" s="17"/>
+      <c r="E18" s="9"/>
     </row>
     <row r="19" spans="3:5">
-      <c r="C19" s="17"/>
-      <c r="D19" s="17" t="s">
+      <c r="C19" s="9"/>
+      <c r="D19" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="E19" s="17"/>
+      <c r="E19" s="9"/>
     </row>
     <row r="20" spans="3:5">
-      <c r="C20" s="17"/>
-      <c r="D20" s="17" t="s">
+      <c r="C20" s="9"/>
+      <c r="D20" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="E20" s="17"/>
+      <c r="E20" s="9"/>
     </row>
     <row r="21" spans="3:5">
-      <c r="C21" s="17"/>
-      <c r="D21" s="17" t="s">
+      <c r="C21" s="9"/>
+      <c r="D21" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="E21" s="17"/>
+      <c r="E21" s="9"/>
     </row>
     <row r="22" spans="3:5">
-      <c r="C22" s="17"/>
-      <c r="D22" s="17" t="s">
+      <c r="C22" s="9"/>
+      <c r="D22" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E22" s="17"/>
+      <c r="E22" s="9"/>
     </row>
     <row r="23" spans="3:5">
-      <c r="C23" s="17"/>
-      <c r="D23" s="17" t="s">
+      <c r="C23" s="9"/>
+      <c r="D23" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="E23" s="17"/>
+      <c r="E23" s="9"/>
     </row>
     <row r="24" spans="3:5">
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
     </row>
     <row r="25" spans="3:3">
-      <c r="C25" s="17" t="s">
+      <c r="C25" s="9" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="26" spans="3:3">
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="9" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="27" ht="27" customHeight="1" spans="1:8">
-      <c r="A27" s="23" t="s">
+      <c r="A27" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
-      <c r="H27" s="23"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
     </row>
     <row r="28" ht="16" customHeight="1" spans="1:8">
-      <c r="A28" s="23"/>
-      <c r="B28" s="23"/>
-      <c r="C28" s="24" t="s">
+      <c r="A28" s="21"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
     </row>
     <row r="29" ht="16" customHeight="1" spans="1:8">
-      <c r="A29" s="25" t="s">
+      <c r="A29" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="C29" s="24"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="21"/>
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:8">
-      <c r="A30" s="24" t="s">
+      <c r="A30" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="B30" s="23"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23"/>
-      <c r="H30" s="23"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:8">
-      <c r="A31" s="25" t="s">
+      <c r="A31" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="B31" s="25" t="s">
+      <c r="B31" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="C31" s="24"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:8">
-      <c r="A32" s="24" t="s">
+      <c r="A32" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="B32" s="23"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="23"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:8">
-      <c r="A33" s="24"/>
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="23"/>
+      <c r="A33" s="22"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="21"/>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:8">
       <c r="A34" s="9" t="s">
@@ -3882,9 +3880,9 @@
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="23"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+      <c r="H34" s="21"/>
     </row>
     <row r="35" ht="16" customHeight="1" spans="1:8">
       <c r="A35" s="9"/>
@@ -3894,9 +3892,9 @@
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
-      <c r="F35" s="24"/>
-      <c r="G35" s="24"/>
-      <c r="H35" s="23"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="22"/>
+      <c r="H35" s="21"/>
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:8">
       <c r="A36" s="10" t="s">
@@ -3908,12 +3906,12 @@
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="24"/>
-      <c r="H36" s="23"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="22"/>
+      <c r="H36" s="21"/>
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:8">
-      <c r="A37" s="24" t="s">
+      <c r="A37" s="22" t="s">
         <v>97</v>
       </c>
       <c r="B37" s="10" t="s">
@@ -3924,9 +3922,9 @@
         <v>99</v>
       </c>
       <c r="E37" s="9"/>
-      <c r="F37" s="24"/>
-      <c r="G37" s="24"/>
-      <c r="H37" s="23"/>
+      <c r="F37" s="22"/>
+      <c r="G37" s="22"/>
+      <c r="H37" s="21"/>
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:8">
       <c r="A38" s="9"/>
@@ -3938,335 +3936,335 @@
         <v>101</v>
       </c>
       <c r="E38" s="9"/>
-      <c r="F38" s="24"/>
-      <c r="G38" s="24"/>
-      <c r="H38" s="23"/>
+      <c r="F38" s="22"/>
+      <c r="G38" s="22"/>
+      <c r="H38" s="21"/>
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:8">
-      <c r="A39" s="24"/>
-      <c r="B39" s="24"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24" t="s">
+      <c r="A39" s="22"/>
+      <c r="B39" s="22"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="E39" s="24"/>
-      <c r="F39" s="24" t="s">
+      <c r="E39" s="22"/>
+      <c r="F39" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="G39" s="24"/>
-      <c r="H39" s="23"/>
+      <c r="G39" s="22"/>
+      <c r="H39" s="21"/>
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:8">
-      <c r="A40" s="24"/>
-      <c r="B40" s="24"/>
-      <c r="C40" s="24" t="s">
+      <c r="A40" s="22"/>
+      <c r="B40" s="22"/>
+      <c r="C40" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="D40" s="24"/>
-      <c r="E40" s="24"/>
-      <c r="F40" s="24"/>
-      <c r="G40" s="24"/>
-      <c r="H40" s="23"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="22"/>
+      <c r="H40" s="21"/>
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:8">
-      <c r="A41" s="24"/>
-      <c r="B41" s="24"/>
-      <c r="C41" s="24" t="s">
+      <c r="A41" s="22"/>
+      <c r="B41" s="22"/>
+      <c r="C41" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="D41" s="24"/>
-      <c r="E41" s="24"/>
-      <c r="F41" s="24"/>
-      <c r="G41" s="24"/>
-      <c r="H41" s="23"/>
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="22"/>
+      <c r="H41" s="21"/>
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:8">
-      <c r="A42" s="24" t="s">
+      <c r="A42" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="B42" s="24" t="s">
+      <c r="B42" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="C42" s="24" t="s">
+      <c r="C42" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="D42" s="24"/>
-      <c r="E42" s="24"/>
-      <c r="F42" s="24"/>
-      <c r="G42" s="24"/>
-      <c r="H42" s="23"/>
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="22"/>
+      <c r="H42" s="21"/>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:8">
-      <c r="A43" s="24"/>
-      <c r="B43" s="24" t="s">
+      <c r="A43" s="22"/>
+      <c r="B43" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
-      <c r="G43" s="24"/>
-      <c r="H43" s="23"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="22"/>
+      <c r="E43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="22"/>
+      <c r="H43" s="21"/>
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:8">
-      <c r="A44" s="24"/>
-      <c r="B44" s="24" t="s">
+      <c r="A44" s="22"/>
+      <c r="B44" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="C44" s="24"/>
-      <c r="D44" s="24"/>
-      <c r="E44" s="24"/>
-      <c r="F44" s="24"/>
-      <c r="G44" s="24"/>
-      <c r="H44" s="23"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
+      <c r="G44" s="22"/>
+      <c r="H44" s="21"/>
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:8">
-      <c r="A45" s="24"/>
-      <c r="B45" s="24"/>
-      <c r="C45" s="24"/>
-      <c r="D45" s="24"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="24"/>
-      <c r="G45" s="24"/>
-      <c r="H45" s="23"/>
+      <c r="A45" s="22"/>
+      <c r="B45" s="22"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="22"/>
+      <c r="H45" s="21"/>
     </row>
     <row r="46" ht="16" customHeight="1" spans="1:8">
-      <c r="A46" s="24"/>
-      <c r="B46" s="24"/>
-      <c r="C46" s="24"/>
-      <c r="D46" s="24"/>
-      <c r="E46" s="24"/>
-      <c r="F46" s="24"/>
-      <c r="G46" s="24"/>
-      <c r="H46" s="23"/>
+      <c r="A46" s="22"/>
+      <c r="B46" s="22"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="22"/>
+      <c r="H46" s="21"/>
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:8">
-      <c r="A47" s="24"/>
-      <c r="B47" s="24"/>
-      <c r="C47" s="24"/>
-      <c r="D47" s="24"/>
-      <c r="E47" s="24"/>
-      <c r="F47" s="24"/>
-      <c r="G47" s="24"/>
-      <c r="H47" s="23"/>
+      <c r="A47" s="22"/>
+      <c r="B47" s="22"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="22"/>
+      <c r="H47" s="21"/>
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:8">
-      <c r="A48" s="24"/>
-      <c r="B48" s="24"/>
-      <c r="C48" s="24"/>
-      <c r="D48" s="24"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="24"/>
-      <c r="G48" s="24"/>
-      <c r="H48" s="23"/>
+      <c r="A48" s="22"/>
+      <c r="B48" s="22"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="22"/>
+      <c r="H48" s="21"/>
     </row>
     <row r="49" ht="16" customHeight="1" spans="1:8">
-      <c r="A49" s="24"/>
-      <c r="B49" s="24"/>
-      <c r="C49" s="24"/>
-      <c r="D49" s="24"/>
-      <c r="E49" s="24"/>
-      <c r="F49" s="24"/>
-      <c r="G49" s="24"/>
-      <c r="H49" s="23"/>
+      <c r="A49" s="22"/>
+      <c r="B49" s="22"/>
+      <c r="C49" s="22"/>
+      <c r="D49" s="22"/>
+      <c r="E49" s="22"/>
+      <c r="F49" s="22"/>
+      <c r="G49" s="22"/>
+      <c r="H49" s="21"/>
     </row>
     <row r="50" ht="16" customHeight="1" spans="1:8">
-      <c r="A50" s="24"/>
-      <c r="B50" s="24"/>
-      <c r="C50" s="24"/>
-      <c r="D50" s="24"/>
-      <c r="E50" s="24"/>
-      <c r="F50" s="24"/>
-      <c r="G50" s="24"/>
-      <c r="H50" s="23"/>
+      <c r="A50" s="22"/>
+      <c r="B50" s="22"/>
+      <c r="C50" s="22"/>
+      <c r="D50" s="22"/>
+      <c r="E50" s="22"/>
+      <c r="F50" s="22"/>
+      <c r="G50" s="22"/>
+      <c r="H50" s="21"/>
     </row>
     <row r="51" ht="16" customHeight="1" spans="1:8">
-      <c r="A51" s="24"/>
-      <c r="B51" s="24"/>
-      <c r="C51" s="24"/>
-      <c r="D51" s="24"/>
-      <c r="E51" s="24"/>
-      <c r="F51" s="24"/>
-      <c r="G51" s="24"/>
-      <c r="H51" s="23"/>
+      <c r="A51" s="22"/>
+      <c r="B51" s="22"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="22"/>
+      <c r="E51" s="22"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="22"/>
+      <c r="H51" s="21"/>
     </row>
     <row r="52" ht="16" customHeight="1" spans="1:8">
-      <c r="A52" s="24"/>
-      <c r="B52" s="24"/>
-      <c r="C52" s="24"/>
-      <c r="D52" s="24"/>
-      <c r="E52" s="24"/>
-      <c r="F52" s="24"/>
-      <c r="G52" s="24"/>
-      <c r="H52" s="23"/>
+      <c r="A52" s="22"/>
+      <c r="B52" s="22"/>
+      <c r="C52" s="22"/>
+      <c r="D52" s="22"/>
+      <c r="E52" s="22"/>
+      <c r="F52" s="22"/>
+      <c r="G52" s="22"/>
+      <c r="H52" s="21"/>
     </row>
     <row r="53" ht="16" customHeight="1" spans="1:8">
-      <c r="A53" s="24"/>
-      <c r="B53" s="24"/>
-      <c r="C53" s="24"/>
-      <c r="D53" s="24"/>
-      <c r="E53" s="24"/>
-      <c r="F53" s="24"/>
-      <c r="G53" s="24"/>
-      <c r="H53" s="23"/>
+      <c r="A53" s="22"/>
+      <c r="B53" s="22"/>
+      <c r="C53" s="22"/>
+      <c r="D53" s="22"/>
+      <c r="E53" s="22"/>
+      <c r="F53" s="22"/>
+      <c r="G53" s="22"/>
+      <c r="H53" s="21"/>
     </row>
     <row r="54" ht="16" customHeight="1" spans="1:8">
-      <c r="A54" s="24"/>
-      <c r="B54" s="24"/>
-      <c r="C54" s="24"/>
-      <c r="D54" s="24"/>
-      <c r="E54" s="24"/>
-      <c r="F54" s="24"/>
-      <c r="G54" s="24"/>
-      <c r="H54" s="23"/>
+      <c r="A54" s="22"/>
+      <c r="B54" s="22"/>
+      <c r="C54" s="22"/>
+      <c r="D54" s="22"/>
+      <c r="E54" s="22"/>
+      <c r="F54" s="22"/>
+      <c r="G54" s="22"/>
+      <c r="H54" s="21"/>
     </row>
     <row r="55" ht="16" customHeight="1" spans="1:8">
-      <c r="A55" s="24"/>
-      <c r="B55" s="24"/>
-      <c r="C55" s="24"/>
-      <c r="D55" s="24"/>
-      <c r="E55" s="24"/>
-      <c r="F55" s="24"/>
-      <c r="G55" s="24"/>
-      <c r="H55" s="23"/>
+      <c r="A55" s="22"/>
+      <c r="B55" s="22"/>
+      <c r="C55" s="22"/>
+      <c r="D55" s="22"/>
+      <c r="E55" s="22"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="22"/>
+      <c r="H55" s="21"/>
     </row>
     <row r="56" ht="16" customHeight="1" spans="1:8">
-      <c r="A56" s="24"/>
-      <c r="B56" s="24"/>
-      <c r="C56" s="24"/>
-      <c r="D56" s="24"/>
-      <c r="E56" s="24"/>
-      <c r="F56" s="24"/>
-      <c r="G56" s="24"/>
-      <c r="H56" s="23"/>
+      <c r="A56" s="22"/>
+      <c r="B56" s="22"/>
+      <c r="C56" s="22"/>
+      <c r="D56" s="22"/>
+      <c r="E56" s="22"/>
+      <c r="F56" s="22"/>
+      <c r="G56" s="22"/>
+      <c r="H56" s="21"/>
     </row>
     <row r="57" ht="16" customHeight="1" spans="1:8">
-      <c r="A57" s="24"/>
-      <c r="B57" s="24"/>
-      <c r="C57" s="24"/>
-      <c r="D57" s="24"/>
-      <c r="E57" s="24"/>
-      <c r="F57" s="24"/>
-      <c r="G57" s="24"/>
-      <c r="H57" s="23"/>
+      <c r="A57" s="22"/>
+      <c r="B57" s="22"/>
+      <c r="C57" s="22"/>
+      <c r="D57" s="22"/>
+      <c r="E57" s="22"/>
+      <c r="F57" s="22"/>
+      <c r="G57" s="22"/>
+      <c r="H57" s="21"/>
     </row>
     <row r="58" ht="16" customHeight="1" spans="1:8">
-      <c r="A58" s="24"/>
-      <c r="B58" s="24"/>
-      <c r="C58" s="24"/>
-      <c r="D58" s="24"/>
-      <c r="E58" s="24"/>
-      <c r="F58" s="24"/>
-      <c r="G58" s="24"/>
-      <c r="H58" s="23"/>
+      <c r="A58" s="22"/>
+      <c r="B58" s="22"/>
+      <c r="C58" s="22"/>
+      <c r="D58" s="22"/>
+      <c r="E58" s="22"/>
+      <c r="F58" s="22"/>
+      <c r="G58" s="22"/>
+      <c r="H58" s="21"/>
     </row>
     <row r="59" ht="16" customHeight="1" spans="1:8">
-      <c r="A59" s="24"/>
-      <c r="B59" s="24"/>
-      <c r="C59" s="24"/>
-      <c r="D59" s="24"/>
-      <c r="E59" s="24"/>
-      <c r="F59" s="24"/>
-      <c r="G59" s="24"/>
-      <c r="H59" s="23"/>
+      <c r="A59" s="22"/>
+      <c r="B59" s="22"/>
+      <c r="C59" s="22"/>
+      <c r="D59" s="22"/>
+      <c r="E59" s="22"/>
+      <c r="F59" s="22"/>
+      <c r="G59" s="22"/>
+      <c r="H59" s="21"/>
     </row>
     <row r="60" ht="16" customHeight="1" spans="1:8">
-      <c r="A60" s="24"/>
-      <c r="B60" s="24"/>
-      <c r="C60" s="24"/>
-      <c r="D60" s="24"/>
-      <c r="E60" s="24"/>
-      <c r="F60" s="24"/>
-      <c r="G60" s="24"/>
-      <c r="H60" s="23"/>
+      <c r="A60" s="22"/>
+      <c r="B60" s="22"/>
+      <c r="C60" s="22"/>
+      <c r="D60" s="22"/>
+      <c r="E60" s="22"/>
+      <c r="F60" s="22"/>
+      <c r="G60" s="22"/>
+      <c r="H60" s="21"/>
     </row>
     <row r="61" ht="16" customHeight="1" spans="1:8">
-      <c r="A61" s="24"/>
-      <c r="B61" s="24"/>
-      <c r="C61" s="24"/>
-      <c r="D61" s="24"/>
-      <c r="E61" s="24"/>
-      <c r="F61" s="24"/>
-      <c r="G61" s="24"/>
-      <c r="H61" s="23"/>
+      <c r="A61" s="22"/>
+      <c r="B61" s="22"/>
+      <c r="C61" s="22"/>
+      <c r="D61" s="22"/>
+      <c r="E61" s="22"/>
+      <c r="F61" s="22"/>
+      <c r="G61" s="22"/>
+      <c r="H61" s="21"/>
     </row>
     <row r="62" ht="16" customHeight="1" spans="1:8">
-      <c r="A62" s="24"/>
-      <c r="B62" s="24"/>
-      <c r="C62" s="24"/>
-      <c r="D62" s="24"/>
-      <c r="E62" s="24"/>
-      <c r="F62" s="24"/>
-      <c r="G62" s="24"/>
-      <c r="H62" s="23"/>
+      <c r="A62" s="22"/>
+      <c r="B62" s="22"/>
+      <c r="C62" s="22"/>
+      <c r="D62" s="22"/>
+      <c r="E62" s="22"/>
+      <c r="F62" s="22"/>
+      <c r="G62" s="22"/>
+      <c r="H62" s="21"/>
     </row>
     <row r="63" ht="16" customHeight="1" spans="1:8">
-      <c r="A63" s="24"/>
-      <c r="B63" s="24"/>
-      <c r="C63" s="24"/>
-      <c r="D63" s="24"/>
-      <c r="E63" s="24"/>
-      <c r="F63" s="24"/>
-      <c r="G63" s="24"/>
-      <c r="H63" s="23"/>
+      <c r="A63" s="22"/>
+      <c r="B63" s="22"/>
+      <c r="C63" s="22"/>
+      <c r="D63" s="22"/>
+      <c r="E63" s="22"/>
+      <c r="F63" s="22"/>
+      <c r="G63" s="22"/>
+      <c r="H63" s="21"/>
     </row>
     <row r="64" ht="16" customHeight="1" spans="1:8">
-      <c r="A64" s="24"/>
-      <c r="B64" s="24"/>
-      <c r="C64" s="24"/>
-      <c r="D64" s="24"/>
-      <c r="E64" s="24"/>
-      <c r="F64" s="24"/>
-      <c r="G64" s="24"/>
-      <c r="H64" s="23"/>
+      <c r="A64" s="22"/>
+      <c r="B64" s="22"/>
+      <c r="C64" s="22"/>
+      <c r="D64" s="22"/>
+      <c r="E64" s="22"/>
+      <c r="F64" s="22"/>
+      <c r="G64" s="22"/>
+      <c r="H64" s="21"/>
     </row>
     <row r="65" ht="16" customHeight="1" spans="1:8">
-      <c r="A65" s="24"/>
-      <c r="B65" s="24"/>
-      <c r="C65" s="24"/>
-      <c r="D65" s="24"/>
-      <c r="E65" s="24"/>
-      <c r="F65" s="24"/>
-      <c r="G65" s="24"/>
-      <c r="H65" s="23"/>
+      <c r="A65" s="22"/>
+      <c r="B65" s="22"/>
+      <c r="C65" s="22"/>
+      <c r="D65" s="22"/>
+      <c r="E65" s="22"/>
+      <c r="F65" s="22"/>
+      <c r="G65" s="22"/>
+      <c r="H65" s="21"/>
     </row>
     <row r="66" ht="16" customHeight="1" spans="1:8">
-      <c r="A66" s="24"/>
-      <c r="B66" s="24"/>
-      <c r="C66" s="24"/>
-      <c r="D66" s="24"/>
-      <c r="E66" s="24"/>
-      <c r="F66" s="24"/>
-      <c r="G66" s="24"/>
-      <c r="H66" s="23"/>
+      <c r="A66" s="22"/>
+      <c r="B66" s="22"/>
+      <c r="C66" s="22"/>
+      <c r="D66" s="22"/>
+      <c r="E66" s="22"/>
+      <c r="F66" s="22"/>
+      <c r="G66" s="22"/>
+      <c r="H66" s="21"/>
     </row>
     <row r="67" ht="16" customHeight="1" spans="1:8">
-      <c r="A67" s="24"/>
-      <c r="B67" s="24"/>
-      <c r="C67" s="24"/>
-      <c r="D67" s="24"/>
-      <c r="E67" s="24"/>
-      <c r="F67" s="24"/>
-      <c r="G67" s="24"/>
-      <c r="H67" s="23"/>
+      <c r="A67" s="22"/>
+      <c r="B67" s="22"/>
+      <c r="C67" s="22"/>
+      <c r="D67" s="22"/>
+      <c r="E67" s="22"/>
+      <c r="F67" s="22"/>
+      <c r="G67" s="22"/>
+      <c r="H67" s="21"/>
     </row>
     <row r="68" ht="16" customHeight="1" spans="1:8">
-      <c r="A68" s="24"/>
-      <c r="B68" s="24"/>
-      <c r="C68" s="24"/>
-      <c r="D68" s="24"/>
-      <c r="E68" s="24"/>
-      <c r="F68" s="24"/>
-      <c r="G68" s="24"/>
-      <c r="H68" s="23"/>
+      <c r="A68" s="22"/>
+      <c r="B68" s="22"/>
+      <c r="C68" s="22"/>
+      <c r="D68" s="22"/>
+      <c r="E68" s="22"/>
+      <c r="F68" s="22"/>
+      <c r="G68" s="22"/>
+      <c r="H68" s="21"/>
     </row>
     <row r="69" spans="1:7">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
-      <c r="C69" s="17" t="s">
+      <c r="C69" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="D69" s="17"/>
+      <c r="D69" s="9"/>
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
@@ -4274,10 +4272,10 @@
     <row r="70" spans="1:7">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
-      <c r="C70" s="17" t="s">
+      <c r="C70" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="D70" s="17"/>
+      <c r="D70" s="9"/>
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -4285,8 +4283,8 @@
     <row r="71" spans="1:7">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
-      <c r="C71" s="17"/>
-      <c r="D71" s="17" t="s">
+      <c r="C71" s="9"/>
+      <c r="D71" s="9" t="s">
         <v>112</v>
       </c>
       <c r="E71" s="3"/>
@@ -4294,20 +4292,20 @@
       <c r="G71" s="3"/>
     </row>
     <row r="72" spans="3:4">
-      <c r="C72" s="17"/>
-      <c r="D72" s="17"/>
+      <c r="C72" s="9"/>
+      <c r="D72" s="9"/>
     </row>
     <row r="73" spans="1:3">
-      <c r="A73" s="26" t="s">
+      <c r="A73" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B73" s="17"/>
-      <c r="C73" s="17" t="s">
+      <c r="B73" s="9"/>
+      <c r="C73" s="9" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="74" spans="1:1">
-      <c r="A74" s="27" t="s">
+      <c r="A74" s="25" t="s">
         <v>115</v>
       </c>
     </row>
@@ -4440,7 +4438,7 @@
       </c>
     </row>
     <row r="16" ht="14.5" spans="2:4">
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="16" t="s">
         <v>129</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -4448,7 +4446,7 @@
       </c>
     </row>
     <row r="17" ht="14.5" spans="2:5">
-      <c r="B17" s="18"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="1" t="s">
         <v>130</v>
       </c>
@@ -4457,34 +4455,34 @@
       </c>
     </row>
     <row r="18" ht="14.5" spans="2:4">
-      <c r="B18" s="18"/>
+      <c r="B18" s="16"/>
       <c r="D18" s="1" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="19" ht="14.5" spans="2:2">
-      <c r="B19" s="18"/>
+      <c r="B19" s="16"/>
     </row>
     <row r="20" ht="14.5" spans="1:3">
       <c r="A20" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B20" s="18"/>
+      <c r="B20" s="16"/>
       <c r="C20" s="1" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="21" ht="14.5" spans="2:2">
-      <c r="B21" s="18"/>
+      <c r="B21" s="16"/>
     </row>
     <row r="22" ht="14.5" spans="2:3">
-      <c r="B22" s="18"/>
+      <c r="B22" s="16"/>
       <c r="C22" s="1" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="23" ht="14.5" spans="2:4">
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="16" t="s">
         <v>135</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -4492,19 +4490,19 @@
       </c>
     </row>
     <row r="24" ht="14.5" spans="2:3">
-      <c r="B24" s="18"/>
+      <c r="B24" s="16"/>
       <c r="C24" s="1" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="25" ht="14.5" spans="2:2">
-      <c r="B25" s="18"/>
+      <c r="B25" s="16"/>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="B26" s="17" t="s">
         <v>138</v>
       </c>
     </row>
@@ -4648,7 +4646,7 @@
       <c r="A47" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D47" s="17" t="s">
+      <c r="D47" s="9" t="s">
         <v>166</v>
       </c>
     </row>
@@ -4775,141 +4773,141 @@
       </c>
     </row>
     <row r="67" spans="3:3">
-      <c r="C67" s="17" t="s">
+      <c r="C67" s="9" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="68" spans="3:4">
-      <c r="C68" s="17"/>
-      <c r="D68" s="17" t="s">
+      <c r="C68" s="9"/>
+      <c r="D68" s="9" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="69" spans="3:5">
-      <c r="C69" s="17"/>
+      <c r="C69" s="9"/>
       <c r="E69" s="1" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="70" spans="3:4">
-      <c r="C70" s="17"/>
+      <c r="C70" s="9"/>
       <c r="D70" s="1" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="71" spans="3:5">
-      <c r="C71" s="17"/>
+      <c r="C71" s="9"/>
       <c r="E71" s="1" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="72" spans="3:4">
-      <c r="C72" s="17"/>
+      <c r="C72" s="9"/>
       <c r="D72" s="1" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="73" spans="3:3">
-      <c r="C73" s="17"/>
+      <c r="C73" s="9"/>
     </row>
     <row r="74" spans="1:6">
-      <c r="A74" s="20"/>
-      <c r="B74" s="20"/>
-      <c r="C74" s="20"/>
-      <c r="D74" s="20"/>
-      <c r="E74" s="20"/>
-      <c r="F74" s="20"/>
+      <c r="A74" s="18"/>
+      <c r="B74" s="18"/>
+      <c r="C74" s="18"/>
+      <c r="D74" s="18"/>
+      <c r="E74" s="18"/>
+      <c r="F74" s="18"/>
     </row>
     <row r="75" spans="1:6">
-      <c r="A75" s="20"/>
-      <c r="B75" s="20"/>
-      <c r="C75" s="20"/>
-      <c r="D75" s="20"/>
-      <c r="E75" s="20"/>
-      <c r="F75" s="20"/>
+      <c r="A75" s="18"/>
+      <c r="B75" s="18"/>
+      <c r="C75" s="18"/>
+      <c r="D75" s="18"/>
+      <c r="E75" s="18"/>
+      <c r="F75" s="18"/>
     </row>
     <row r="76" spans="1:6">
-      <c r="A76" s="20"/>
-      <c r="B76" s="20"/>
-      <c r="C76" s="20"/>
-      <c r="D76" s="20"/>
-      <c r="E76" s="20"/>
-      <c r="F76" s="20"/>
+      <c r="A76" s="18"/>
+      <c r="B76" s="18"/>
+      <c r="C76" s="18"/>
+      <c r="D76" s="18"/>
+      <c r="E76" s="18"/>
+      <c r="F76" s="18"/>
     </row>
     <row r="77" spans="1:6">
-      <c r="A77" s="20"/>
-      <c r="B77" s="20"/>
-      <c r="C77" s="20"/>
-      <c r="D77" s="20"/>
-      <c r="E77" s="20"/>
-      <c r="F77" s="20"/>
+      <c r="A77" s="18"/>
+      <c r="B77" s="18"/>
+      <c r="C77" s="18"/>
+      <c r="D77" s="18"/>
+      <c r="E77" s="18"/>
+      <c r="F77" s="18"/>
     </row>
     <row r="78" spans="1:6">
-      <c r="A78" s="20"/>
-      <c r="B78" s="20"/>
-      <c r="C78" s="20"/>
-      <c r="D78" s="20"/>
-      <c r="E78" s="20"/>
-      <c r="F78" s="20"/>
+      <c r="A78" s="18"/>
+      <c r="B78" s="18"/>
+      <c r="C78" s="18"/>
+      <c r="D78" s="18"/>
+      <c r="E78" s="18"/>
+      <c r="F78" s="18"/>
     </row>
     <row r="79" spans="1:6">
-      <c r="A79" s="20"/>
-      <c r="B79" s="20"/>
-      <c r="C79" s="20"/>
-      <c r="D79" s="20"/>
-      <c r="E79" s="20"/>
-      <c r="F79" s="20"/>
+      <c r="A79" s="18"/>
+      <c r="B79" s="18"/>
+      <c r="C79" s="18"/>
+      <c r="D79" s="18"/>
+      <c r="E79" s="18"/>
+      <c r="F79" s="18"/>
     </row>
     <row r="80" spans="1:6">
-      <c r="A80" s="20"/>
-      <c r="B80" s="20"/>
-      <c r="C80" s="20"/>
-      <c r="D80" s="20"/>
-      <c r="E80" s="20"/>
-      <c r="F80" s="20"/>
+      <c r="A80" s="18"/>
+      <c r="B80" s="18"/>
+      <c r="C80" s="18"/>
+      <c r="D80" s="18"/>
+      <c r="E80" s="18"/>
+      <c r="F80" s="18"/>
     </row>
     <row r="81" spans="1:6">
-      <c r="A81" s="20"/>
-      <c r="B81" s="20"/>
-      <c r="C81" s="20"/>
-      <c r="D81" s="20"/>
-      <c r="E81" s="20"/>
-      <c r="F81" s="20"/>
+      <c r="A81" s="18"/>
+      <c r="B81" s="18"/>
+      <c r="C81" s="18"/>
+      <c r="D81" s="18"/>
+      <c r="E81" s="18"/>
+      <c r="F81" s="18"/>
     </row>
     <row r="82" spans="1:6">
-      <c r="A82" s="20"/>
-      <c r="B82" s="20"/>
-      <c r="C82" s="20"/>
-      <c r="D82" s="20"/>
-      <c r="E82" s="20"/>
-      <c r="F82" s="20"/>
+      <c r="A82" s="18"/>
+      <c r="B82" s="18"/>
+      <c r="C82" s="18"/>
+      <c r="D82" s="18"/>
+      <c r="E82" s="18"/>
+      <c r="F82" s="18"/>
     </row>
     <row r="93" spans="3:4">
-      <c r="C93" s="17"/>
-      <c r="D93" s="17"/>
+      <c r="C93" s="9"/>
+      <c r="D93" s="9"/>
     </row>
     <row r="94" spans="3:4">
-      <c r="C94" s="17"/>
-      <c r="D94" s="17"/>
+      <c r="C94" s="9"/>
+      <c r="D94" s="9"/>
     </row>
     <row r="95" spans="3:4">
-      <c r="C95" s="17"/>
-      <c r="D95" s="17"/>
+      <c r="C95" s="9"/>
+      <c r="D95" s="9"/>
     </row>
     <row r="96" spans="3:4">
-      <c r="C96" s="17"/>
-      <c r="D96" s="17"/>
+      <c r="C96" s="9"/>
+      <c r="D96" s="9"/>
     </row>
     <row r="97" spans="3:4">
-      <c r="C97" s="17"/>
-      <c r="D97" s="17"/>
+      <c r="C97" s="9"/>
+      <c r="D97" s="9"/>
     </row>
     <row r="98" spans="4:4">
-      <c r="D98" s="17"/>
+      <c r="D98" s="9"/>
     </row>
     <row r="99" spans="3:4">
-      <c r="C99" s="17"/>
-      <c r="D99" s="17"/>
+      <c r="C99" s="9"/>
+      <c r="D99" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5003,7 +5001,7 @@
     <col min="4" max="4" width="3.33076923076923" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.6692307692308" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.1692307692308" style="1" customWidth="1"/>
-    <col min="7" max="7" width="4.5" style="16" customWidth="1"/>
+    <col min="7" max="7" width="4.5" style="15" customWidth="1"/>
     <col min="8" max="8" width="4.5" style="1" customWidth="1"/>
     <col min="9" max="16384" width="8.66923076923077" style="1"/>
   </cols>
@@ -5131,118 +5129,118 @@
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="17"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17" t="s">
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="17"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17" t="s">
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17" t="s">
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="17"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17" t="s">
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="F22" s="17"/>
+      <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17" t="s">
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="F23" s="17"/>
+      <c r="F23" s="9"/>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17" t="s">
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="F24" s="17"/>
+      <c r="F24" s="9"/>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="17"/>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17" t="s">
+      <c r="A25" s="9"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17" t="s">
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="17" t="s">
+      <c r="A27" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="17" t="s">
+      <c r="A28" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
     </row>
     <row r="29" ht="15.5" spans="1:5">
       <c r="A29"/>
@@ -5306,7 +5304,7 @@
       <c r="D36" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="G36" s="16">
+      <c r="G36" s="15">
         <v>5</v>
       </c>
     </row>
@@ -5396,46 +5394,46 @@
       </c>
     </row>
     <row r="3" spans="3:5">
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
     </row>
     <row r="4" spans="3:5">
-      <c r="C4" s="15"/>
-      <c r="D4" s="15" t="s">
+      <c r="C4" s="10"/>
+      <c r="D4" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="E4" s="15"/>
+      <c r="E4" s="10"/>
     </row>
     <row r="5" spans="3:5">
-      <c r="C5" s="15"/>
+      <c r="C5" s="10"/>
       <c r="D5" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="E5" s="15"/>
+      <c r="E5" s="10"/>
     </row>
     <row r="6" spans="3:5">
-      <c r="C6" s="15"/>
+      <c r="C6" s="10"/>
       <c r="D6" s="12" t="s">
         <v>257</v>
       </c>
-      <c r="E6" s="15"/>
+      <c r="E6" s="10"/>
     </row>
     <row r="7" spans="3:5">
-      <c r="C7" s="15"/>
+      <c r="C7" s="10"/>
       <c r="D7" s="12" t="s">
         <v>258</v>
       </c>
-      <c r="E7" s="15"/>
+      <c r="E7" s="10"/>
     </row>
     <row r="8" spans="3:5">
-      <c r="C8" s="15"/>
-      <c r="D8" s="15" t="s">
+      <c r="C8" s="10"/>
+      <c r="D8" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="E8" s="15"/>
+      <c r="E8" s="10"/>
     </row>
     <row r="9" spans="4:4">
       <c r="D9" s="12" t="s">
@@ -5443,12 +5441,12 @@
       </c>
     </row>
     <row r="10" spans="4:4">
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="10" t="s">
         <v>261</v>
       </c>
     </row>
     <row r="11" spans="4:4">
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="10" t="s">
         <v>262</v>
       </c>
     </row>
@@ -5605,42 +5603,42 @@
       </c>
     </row>
     <row r="35" spans="3:4">
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="D35" s="15"/>
+      <c r="D35" s="10"/>
     </row>
     <row r="36" spans="3:4">
-      <c r="C36" s="15"/>
-      <c r="D36" s="15" t="s">
+      <c r="C36" s="10"/>
+      <c r="D36" s="10" t="s">
         <v>297</v>
       </c>
     </row>
     <row r="37" spans="3:4">
-      <c r="C37" s="15"/>
-      <c r="D37" s="15" t="s">
+      <c r="C37" s="10"/>
+      <c r="D37" s="10" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="38" spans="3:4">
-      <c r="C38" s="15" t="s">
+      <c r="C38" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="D38" s="15"/>
+      <c r="D38" s="10"/>
     </row>
     <row r="39" spans="3:4">
-      <c r="C39" s="15"/>
-      <c r="D39" s="15"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
     </row>
     <row r="40" spans="3:4">
-      <c r="C40" s="15" t="s">
+      <c r="C40" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="D40" s="15"/>
+      <c r="D40" s="10"/>
     </row>
     <row r="41" spans="3:4">
-      <c r="C41" s="15"/>
-      <c r="D41" s="15" t="s">
+      <c r="C41" s="10"/>
+      <c r="D41" s="10" t="s">
         <v>301</v>
       </c>
     </row>

</xml_diff>

<commit_message>
remove waste pandas git ex files
</commit_message>
<xml_diff>
--- a/p/py-25/py-core/topic-list_py.xlsx
+++ b/p/py-25/py-core/topic-list_py.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12200" tabRatio="698" firstSheet="1" activeTab="9"/>
+    <workbookView windowWidth="28800" windowHeight="12200" tabRatio="698" firstSheet="1" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="core" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="495">
   <si>
     <t>Most basic things in py</t>
   </si>
@@ -1344,6 +1344,18 @@
   </si>
   <si>
     <t>http server</t>
+  </si>
+  <si>
+    <t>records</t>
+  </si>
+  <si>
+    <t>Database support includes RedShift, Postgres, MySQL, SQLite, Oracle, and MS-SQL (drivers not included)</t>
+  </si>
+  <si>
+    <t>KDEpy</t>
+  </si>
+  <si>
+    <t>Kernel Density Estimators</t>
   </si>
   <si>
     <t>https://www.quora.com/What-are-the-best-frameworks-for-ETL-processing-using-Python</t>
@@ -2490,7 +2502,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2510,10 +2522,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2907,7 +2922,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="13" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -2918,22 +2933,22 @@
       <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="11"/>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" spans="4:7">
       <c r="D4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="11"/>
+      <c r="G4" s="13"/>
     </row>
     <row r="5" spans="4:7">
       <c r="D5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="11"/>
+      <c r="G5" s="13"/>
     </row>
     <row r="6" spans="7:7">
-      <c r="G6" s="11"/>
+      <c r="G6" s="13"/>
     </row>
     <row r="7" spans="3:3">
       <c r="C7" s="1" t="s">
@@ -2969,16 +2984,16 @@
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:8">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
     </row>
     <row r="16" spans="3:3">
       <c r="C16" s="1" t="s">
@@ -3073,17 +3088,17 @@
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17" t="s">
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="18" t="s">
         <v>41</v>
       </c>
       <c r="D34" s="1" t="s">
@@ -3091,7 +3106,7 @@
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -3099,7 +3114,7 @@
       </c>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" s="17"/>
+      <c r="A36" s="18"/>
     </row>
     <row r="37" spans="3:3">
       <c r="C37" s="1" t="s">
@@ -3107,7 +3122,7 @@
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="17" t="s">
+      <c r="A38" s="18" t="s">
         <v>46</v>
       </c>
       <c r="B38" s="1" t="s">
@@ -3133,9 +3148,9 @@
       </c>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" s="18"/>
-      <c r="B43" s="18"/>
-      <c r="C43" s="18"/>
+      <c r="A43" s="19"/>
+      <c r="B43" s="19"/>
+      <c r="C43" s="19"/>
       <c r="D43" s="1" t="s">
         <v>52</v>
       </c>
@@ -3187,59 +3202,59 @@
       </c>
     </row>
     <row r="53" spans="3:5">
-      <c r="C53" s="18"/>
-      <c r="D53" s="18"/>
-      <c r="E53" s="18"/>
+      <c r="C53" s="19"/>
+      <c r="D53" s="19"/>
+      <c r="E53" s="19"/>
     </row>
     <row r="54" spans="3:5">
-      <c r="C54" s="18"/>
-      <c r="D54" s="18"/>
-      <c r="E54" s="18"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="19"/>
+      <c r="E54" s="19"/>
     </row>
     <row r="55" spans="3:5">
-      <c r="C55" s="18"/>
-      <c r="D55" s="18"/>
-      <c r="E55" s="18"/>
+      <c r="C55" s="19"/>
+      <c r="D55" s="19"/>
+      <c r="E55" s="19"/>
     </row>
     <row r="56" spans="3:5">
-      <c r="C56" s="18"/>
-      <c r="D56" s="18"/>
-      <c r="E56" s="18"/>
+      <c r="C56" s="19"/>
+      <c r="D56" s="19"/>
+      <c r="E56" s="19"/>
     </row>
     <row r="57" spans="3:5">
-      <c r="C57" s="18"/>
-      <c r="D57" s="18"/>
-      <c r="E57" s="18"/>
+      <c r="C57" s="19"/>
+      <c r="D57" s="19"/>
+      <c r="E57" s="19"/>
     </row>
     <row r="58" spans="3:5">
-      <c r="C58" s="18"/>
-      <c r="D58" s="18"/>
-      <c r="E58" s="18"/>
+      <c r="C58" s="19"/>
+      <c r="D58" s="19"/>
+      <c r="E58" s="19"/>
     </row>
     <row r="59" spans="3:5">
-      <c r="C59" s="18"/>
-      <c r="D59" s="18"/>
-      <c r="E59" s="18"/>
+      <c r="C59" s="19"/>
+      <c r="D59" s="19"/>
+      <c r="E59" s="19"/>
     </row>
     <row r="60" spans="3:5">
-      <c r="C60" s="18"/>
-      <c r="D60" s="18"/>
-      <c r="E60" s="18"/>
+      <c r="C60" s="19"/>
+      <c r="D60" s="19"/>
+      <c r="E60" s="19"/>
     </row>
     <row r="61" spans="3:5">
-      <c r="C61" s="18"/>
-      <c r="D61" s="18"/>
-      <c r="E61" s="18"/>
+      <c r="C61" s="19"/>
+      <c r="D61" s="19"/>
+      <c r="E61" s="19"/>
     </row>
     <row r="62" spans="3:5">
-      <c r="C62" s="18"/>
-      <c r="D62" s="18"/>
-      <c r="E62" s="18"/>
+      <c r="C62" s="19"/>
+      <c r="D62" s="19"/>
+      <c r="E62" s="19"/>
     </row>
     <row r="63" spans="3:5">
-      <c r="C63" s="18"/>
-      <c r="D63" s="18"/>
-      <c r="E63" s="18"/>
+      <c r="C63" s="19"/>
+      <c r="D63" s="19"/>
+      <c r="E63" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3262,12 +3277,12 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="2" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
     </row>
     <row r="3" spans="1:1">
@@ -3275,7 +3290,7 @@
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="4" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
     </row>
     <row r="5" spans="1:1">
@@ -3283,32 +3298,32 @@
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="5" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="5" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="6" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="6" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="6" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="5" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="12" spans="1:1">
@@ -3316,7 +3331,7 @@
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="4" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
     </row>
     <row r="14" spans="1:1">
@@ -3324,32 +3339,32 @@
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="5" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="5" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="6" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="5" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
     </row>
     <row r="21" spans="1:1">
@@ -3357,51 +3372,51 @@
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="4" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="3" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="3"/>
       <c r="B24" s="1" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" s="5" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" s="5" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" s="6" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" s="6" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" s="6" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" s="5" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
     </row>
     <row r="31" spans="1:1">
@@ -3409,7 +3424,7 @@
     </row>
     <row r="32" spans="1:1">
       <c r="A32" s="4" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
     </row>
     <row r="33" spans="1:1">
@@ -3417,32 +3432,32 @@
     </row>
     <row r="34" spans="1:1">
       <c r="A34" s="5" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" s="5" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" s="6" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" s="6" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" s="6" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" s="5" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
     </row>
     <row r="40" spans="1:1">
@@ -3450,7 +3465,7 @@
     </row>
     <row r="41" spans="1:1">
       <c r="A41" s="4" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
     </row>
     <row r="42" spans="1:1">
@@ -3458,32 +3473,32 @@
     </row>
     <row r="43" spans="1:1">
       <c r="A43" s="5" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" s="5" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" s="6" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" s="6" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" s="6" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" s="5" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
     </row>
     <row r="49" spans="1:1">
@@ -3491,7 +3506,7 @@
     </row>
     <row r="50" spans="1:1">
       <c r="A50" s="4" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
     </row>
     <row r="51" spans="1:1">
@@ -3499,32 +3514,32 @@
     </row>
     <row r="52" spans="1:1">
       <c r="A52" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
     </row>
     <row r="53" spans="1:1">
       <c r="A53" s="5" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" s="6" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
     </row>
     <row r="55" spans="1:1">
       <c r="A55" s="6" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="56" spans="1:1">
       <c r="A56" s="6" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
     </row>
     <row r="57" spans="1:1">
       <c r="A57" s="5" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
     </row>
     <row r="58" spans="1:1">
@@ -3532,7 +3547,7 @@
     </row>
     <row r="59" spans="1:1">
       <c r="A59" s="4" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
     </row>
     <row r="60" spans="1:1">
@@ -3540,32 +3555,32 @@
     </row>
     <row r="61" spans="1:1">
       <c r="A61" s="5" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
     </row>
     <row r="62" spans="1:1">
       <c r="A62" s="5" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
     </row>
     <row r="63" spans="1:1">
       <c r="A63" s="6" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
     </row>
     <row r="64" spans="1:1">
       <c r="A64" s="6" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
     </row>
     <row r="65" spans="1:1">
       <c r="A65" s="6" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
     </row>
     <row r="66" spans="1:1">
       <c r="A66" s="5" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
     </row>
     <row r="67" spans="1:1">
@@ -3573,37 +3588,37 @@
     </row>
     <row r="68" spans="1:1">
       <c r="A68" s="4" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
     </row>
     <row r="69" spans="1:1">
       <c r="A69" s="2" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
     </row>
     <row r="70" spans="1:1">
       <c r="A70" s="1" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
     <row r="71" spans="1:1">
       <c r="A71" s="1" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
     </row>
     <row r="73" spans="1:1">
       <c r="A73" s="7" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
     </row>
     <row r="74" spans="1:1">
       <c r="A74" s="1" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
     </row>
     <row r="75" spans="1:1">
       <c r="A75" s="1" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
     </row>
   </sheetData>
@@ -3646,7 +3661,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="13" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -3674,7 +3689,7 @@
       </c>
     </row>
     <row r="9" spans="3:3">
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="20" t="s">
         <v>68</v>
       </c>
     </row>
@@ -3687,7 +3702,7 @@
     </row>
     <row r="12" spans="3:5">
       <c r="C12" s="9"/>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="21" t="s">
         <v>70</v>
       </c>
       <c r="E12" s="9"/>
@@ -3788,87 +3803,87 @@
       </c>
     </row>
     <row r="27" ht="27" customHeight="1" spans="1:8">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="B27" s="21"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="21"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
     </row>
     <row r="28" ht="16" customHeight="1" spans="1:8">
-      <c r="A28" s="21"/>
-      <c r="B28" s="21"/>
-      <c r="C28" s="22" t="s">
+      <c r="A28" s="22"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
     </row>
     <row r="29" ht="16" customHeight="1" spans="1:8">
-      <c r="A29" s="23" t="s">
+      <c r="A29" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="C29" s="22"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="21"/>
-      <c r="F29" s="21"/>
-      <c r="G29" s="21"/>
-      <c r="H29" s="21"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:8">
-      <c r="A30" s="22" t="s">
+      <c r="A30" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="B30" s="21"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:8">
-      <c r="A31" s="23" t="s">
+      <c r="A31" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="B31" s="23" t="s">
+      <c r="B31" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="21"/>
+      <c r="C31" s="23"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:8">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B32" s="21"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:8">
-      <c r="A33" s="22"/>
-      <c r="B33" s="22"/>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="22"/>
-      <c r="H33" s="21"/>
+      <c r="A33" s="23"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="22"/>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:8">
       <c r="A34" s="9" t="s">
@@ -3880,9 +3895,9 @@
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="21"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="22"/>
     </row>
     <row r="35" ht="16" customHeight="1" spans="1:8">
       <c r="A35" s="9"/>
@@ -3892,9 +3907,9 @@
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="22"/>
-      <c r="H35" s="21"/>
+      <c r="F35" s="23"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="22"/>
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:8">
       <c r="A36" s="10" t="s">
@@ -3906,12 +3921,12 @@
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="21"/>
+      <c r="F36" s="23"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="22"/>
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:8">
-      <c r="A37" s="22" t="s">
+      <c r="A37" s="23" t="s">
         <v>97</v>
       </c>
       <c r="B37" s="10" t="s">
@@ -3922,9 +3937,9 @@
         <v>99</v>
       </c>
       <c r="E37" s="9"/>
-      <c r="F37" s="22"/>
-      <c r="G37" s="22"/>
-      <c r="H37" s="21"/>
+      <c r="F37" s="23"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="22"/>
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:8">
       <c r="A38" s="9"/>
@@ -3936,327 +3951,327 @@
         <v>101</v>
       </c>
       <c r="E38" s="9"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="21"/>
+      <c r="F38" s="23"/>
+      <c r="G38" s="23"/>
+      <c r="H38" s="22"/>
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:8">
-      <c r="A39" s="22"/>
-      <c r="B39" s="22"/>
-      <c r="C39" s="22"/>
-      <c r="D39" s="22" t="s">
+      <c r="A39" s="23"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="E39" s="22"/>
-      <c r="F39" s="22" t="s">
+      <c r="E39" s="23"/>
+      <c r="F39" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="G39" s="22"/>
-      <c r="H39" s="21"/>
+      <c r="G39" s="23"/>
+      <c r="H39" s="22"/>
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:8">
-      <c r="A40" s="22"/>
-      <c r="B40" s="22"/>
-      <c r="C40" s="22" t="s">
+      <c r="A40" s="23"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="D40" s="22"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="21"/>
+      <c r="D40" s="23"/>
+      <c r="E40" s="23"/>
+      <c r="F40" s="23"/>
+      <c r="G40" s="23"/>
+      <c r="H40" s="22"/>
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:8">
-      <c r="A41" s="22"/>
-      <c r="B41" s="22"/>
-      <c r="C41" s="22" t="s">
+      <c r="A41" s="23"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="D41" s="22"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="21"/>
+      <c r="D41" s="23"/>
+      <c r="E41" s="23"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="22"/>
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:8">
-      <c r="A42" s="22" t="s">
+      <c r="A42" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="B42" s="22" t="s">
+      <c r="B42" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="C42" s="22" t="s">
+      <c r="C42" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="D42" s="22"/>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="21"/>
+      <c r="D42" s="23"/>
+      <c r="E42" s="23"/>
+      <c r="F42" s="23"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="22"/>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:8">
-      <c r="A43" s="22"/>
-      <c r="B43" s="22" t="s">
+      <c r="A43" s="23"/>
+      <c r="B43" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="C43" s="22"/>
-      <c r="D43" s="22"/>
-      <c r="E43" s="22"/>
-      <c r="F43" s="22"/>
-      <c r="G43" s="22"/>
-      <c r="H43" s="21"/>
+      <c r="C43" s="23"/>
+      <c r="D43" s="23"/>
+      <c r="E43" s="23"/>
+      <c r="F43" s="23"/>
+      <c r="G43" s="23"/>
+      <c r="H43" s="22"/>
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:8">
-      <c r="A44" s="22"/>
-      <c r="B44" s="22" t="s">
+      <c r="A44" s="23"/>
+      <c r="B44" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="C44" s="22"/>
-      <c r="D44" s="22"/>
-      <c r="E44" s="22"/>
-      <c r="F44" s="22"/>
-      <c r="G44" s="22"/>
-      <c r="H44" s="21"/>
+      <c r="C44" s="23"/>
+      <c r="D44" s="23"/>
+      <c r="E44" s="23"/>
+      <c r="F44" s="23"/>
+      <c r="G44" s="23"/>
+      <c r="H44" s="22"/>
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:8">
-      <c r="A45" s="22"/>
-      <c r="B45" s="22"/>
-      <c r="C45" s="22"/>
-      <c r="D45" s="22"/>
-      <c r="E45" s="22"/>
-      <c r="F45" s="22"/>
-      <c r="G45" s="22"/>
-      <c r="H45" s="21"/>
+      <c r="A45" s="23"/>
+      <c r="B45" s="23"/>
+      <c r="C45" s="23"/>
+      <c r="D45" s="23"/>
+      <c r="E45" s="23"/>
+      <c r="F45" s="23"/>
+      <c r="G45" s="23"/>
+      <c r="H45" s="22"/>
     </row>
     <row r="46" ht="16" customHeight="1" spans="1:8">
-      <c r="A46" s="22"/>
-      <c r="B46" s="22"/>
-      <c r="C46" s="22"/>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
-      <c r="G46" s="22"/>
-      <c r="H46" s="21"/>
+      <c r="A46" s="23"/>
+      <c r="B46" s="23"/>
+      <c r="C46" s="23"/>
+      <c r="D46" s="23"/>
+      <c r="E46" s="23"/>
+      <c r="F46" s="23"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="22"/>
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:8">
-      <c r="A47" s="22"/>
-      <c r="B47" s="22"/>
-      <c r="C47" s="22"/>
-      <c r="D47" s="22"/>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="22"/>
-      <c r="H47" s="21"/>
+      <c r="A47" s="23"/>
+      <c r="B47" s="23"/>
+      <c r="C47" s="23"/>
+      <c r="D47" s="23"/>
+      <c r="E47" s="23"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="23"/>
+      <c r="H47" s="22"/>
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:8">
-      <c r="A48" s="22"/>
-      <c r="B48" s="22"/>
-      <c r="C48" s="22"/>
-      <c r="D48" s="22"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="22"/>
-      <c r="H48" s="21"/>
+      <c r="A48" s="23"/>
+      <c r="B48" s="23"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="23"/>
+      <c r="E48" s="23"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="23"/>
+      <c r="H48" s="22"/>
     </row>
     <row r="49" ht="16" customHeight="1" spans="1:8">
-      <c r="A49" s="22"/>
-      <c r="B49" s="22"/>
-      <c r="C49" s="22"/>
-      <c r="D49" s="22"/>
-      <c r="E49" s="22"/>
-      <c r="F49" s="22"/>
-      <c r="G49" s="22"/>
-      <c r="H49" s="21"/>
+      <c r="A49" s="23"/>
+      <c r="B49" s="23"/>
+      <c r="C49" s="23"/>
+      <c r="D49" s="23"/>
+      <c r="E49" s="23"/>
+      <c r="F49" s="23"/>
+      <c r="G49" s="23"/>
+      <c r="H49" s="22"/>
     </row>
     <row r="50" ht="16" customHeight="1" spans="1:8">
-      <c r="A50" s="22"/>
-      <c r="B50" s="22"/>
-      <c r="C50" s="22"/>
-      <c r="D50" s="22"/>
-      <c r="E50" s="22"/>
-      <c r="F50" s="22"/>
-      <c r="G50" s="22"/>
-      <c r="H50" s="21"/>
+      <c r="A50" s="23"/>
+      <c r="B50" s="23"/>
+      <c r="C50" s="23"/>
+      <c r="D50" s="23"/>
+      <c r="E50" s="23"/>
+      <c r="F50" s="23"/>
+      <c r="G50" s="23"/>
+      <c r="H50" s="22"/>
     </row>
     <row r="51" ht="16" customHeight="1" spans="1:8">
-      <c r="A51" s="22"/>
-      <c r="B51" s="22"/>
-      <c r="C51" s="22"/>
-      <c r="D51" s="22"/>
-      <c r="E51" s="22"/>
-      <c r="F51" s="22"/>
-      <c r="G51" s="22"/>
-      <c r="H51" s="21"/>
+      <c r="A51" s="23"/>
+      <c r="B51" s="23"/>
+      <c r="C51" s="23"/>
+      <c r="D51" s="23"/>
+      <c r="E51" s="23"/>
+      <c r="F51" s="23"/>
+      <c r="G51" s="23"/>
+      <c r="H51" s="22"/>
     </row>
     <row r="52" ht="16" customHeight="1" spans="1:8">
-      <c r="A52" s="22"/>
-      <c r="B52" s="22"/>
-      <c r="C52" s="22"/>
-      <c r="D52" s="22"/>
-      <c r="E52" s="22"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="22"/>
-      <c r="H52" s="21"/>
+      <c r="A52" s="23"/>
+      <c r="B52" s="23"/>
+      <c r="C52" s="23"/>
+      <c r="D52" s="23"/>
+      <c r="E52" s="23"/>
+      <c r="F52" s="23"/>
+      <c r="G52" s="23"/>
+      <c r="H52" s="22"/>
     </row>
     <row r="53" ht="16" customHeight="1" spans="1:8">
-      <c r="A53" s="22"/>
-      <c r="B53" s="22"/>
-      <c r="C53" s="22"/>
-      <c r="D53" s="22"/>
-      <c r="E53" s="22"/>
-      <c r="F53" s="22"/>
-      <c r="G53" s="22"/>
-      <c r="H53" s="21"/>
+      <c r="A53" s="23"/>
+      <c r="B53" s="23"/>
+      <c r="C53" s="23"/>
+      <c r="D53" s="23"/>
+      <c r="E53" s="23"/>
+      <c r="F53" s="23"/>
+      <c r="G53" s="23"/>
+      <c r="H53" s="22"/>
     </row>
     <row r="54" ht="16" customHeight="1" spans="1:8">
-      <c r="A54" s="22"/>
-      <c r="B54" s="22"/>
-      <c r="C54" s="22"/>
-      <c r="D54" s="22"/>
-      <c r="E54" s="22"/>
-      <c r="F54" s="22"/>
-      <c r="G54" s="22"/>
-      <c r="H54" s="21"/>
+      <c r="A54" s="23"/>
+      <c r="B54" s="23"/>
+      <c r="C54" s="23"/>
+      <c r="D54" s="23"/>
+      <c r="E54" s="23"/>
+      <c r="F54" s="23"/>
+      <c r="G54" s="23"/>
+      <c r="H54" s="22"/>
     </row>
     <row r="55" ht="16" customHeight="1" spans="1:8">
-      <c r="A55" s="22"/>
-      <c r="B55" s="22"/>
-      <c r="C55" s="22"/>
-      <c r="D55" s="22"/>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
-      <c r="G55" s="22"/>
-      <c r="H55" s="21"/>
+      <c r="A55" s="23"/>
+      <c r="B55" s="23"/>
+      <c r="C55" s="23"/>
+      <c r="D55" s="23"/>
+      <c r="E55" s="23"/>
+      <c r="F55" s="23"/>
+      <c r="G55" s="23"/>
+      <c r="H55" s="22"/>
     </row>
     <row r="56" ht="16" customHeight="1" spans="1:8">
-      <c r="A56" s="22"/>
-      <c r="B56" s="22"/>
-      <c r="C56" s="22"/>
-      <c r="D56" s="22"/>
-      <c r="E56" s="22"/>
-      <c r="F56" s="22"/>
-      <c r="G56" s="22"/>
-      <c r="H56" s="21"/>
+      <c r="A56" s="23"/>
+      <c r="B56" s="23"/>
+      <c r="C56" s="23"/>
+      <c r="D56" s="23"/>
+      <c r="E56" s="23"/>
+      <c r="F56" s="23"/>
+      <c r="G56" s="23"/>
+      <c r="H56" s="22"/>
     </row>
     <row r="57" ht="16" customHeight="1" spans="1:8">
-      <c r="A57" s="22"/>
-      <c r="B57" s="22"/>
-      <c r="C57" s="22"/>
-      <c r="D57" s="22"/>
-      <c r="E57" s="22"/>
-      <c r="F57" s="22"/>
-      <c r="G57" s="22"/>
-      <c r="H57" s="21"/>
+      <c r="A57" s="23"/>
+      <c r="B57" s="23"/>
+      <c r="C57" s="23"/>
+      <c r="D57" s="23"/>
+      <c r="E57" s="23"/>
+      <c r="F57" s="23"/>
+      <c r="G57" s="23"/>
+      <c r="H57" s="22"/>
     </row>
     <row r="58" ht="16" customHeight="1" spans="1:8">
-      <c r="A58" s="22"/>
-      <c r="B58" s="22"/>
-      <c r="C58" s="22"/>
-      <c r="D58" s="22"/>
-      <c r="E58" s="22"/>
-      <c r="F58" s="22"/>
-      <c r="G58" s="22"/>
-      <c r="H58" s="21"/>
+      <c r="A58" s="23"/>
+      <c r="B58" s="23"/>
+      <c r="C58" s="23"/>
+      <c r="D58" s="23"/>
+      <c r="E58" s="23"/>
+      <c r="F58" s="23"/>
+      <c r="G58" s="23"/>
+      <c r="H58" s="22"/>
     </row>
     <row r="59" ht="16" customHeight="1" spans="1:8">
-      <c r="A59" s="22"/>
-      <c r="B59" s="22"/>
-      <c r="C59" s="22"/>
-      <c r="D59" s="22"/>
-      <c r="E59" s="22"/>
-      <c r="F59" s="22"/>
-      <c r="G59" s="22"/>
-      <c r="H59" s="21"/>
+      <c r="A59" s="23"/>
+      <c r="B59" s="23"/>
+      <c r="C59" s="23"/>
+      <c r="D59" s="23"/>
+      <c r="E59" s="23"/>
+      <c r="F59" s="23"/>
+      <c r="G59" s="23"/>
+      <c r="H59" s="22"/>
     </row>
     <row r="60" ht="16" customHeight="1" spans="1:8">
-      <c r="A60" s="22"/>
-      <c r="B60" s="22"/>
-      <c r="C60" s="22"/>
-      <c r="D60" s="22"/>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
-      <c r="G60" s="22"/>
-      <c r="H60" s="21"/>
+      <c r="A60" s="23"/>
+      <c r="B60" s="23"/>
+      <c r="C60" s="23"/>
+      <c r="D60" s="23"/>
+      <c r="E60" s="23"/>
+      <c r="F60" s="23"/>
+      <c r="G60" s="23"/>
+      <c r="H60" s="22"/>
     </row>
     <row r="61" ht="16" customHeight="1" spans="1:8">
-      <c r="A61" s="22"/>
-      <c r="B61" s="22"/>
-      <c r="C61" s="22"/>
-      <c r="D61" s="22"/>
-      <c r="E61" s="22"/>
-      <c r="F61" s="22"/>
-      <c r="G61" s="22"/>
-      <c r="H61" s="21"/>
+      <c r="A61" s="23"/>
+      <c r="B61" s="23"/>
+      <c r="C61" s="23"/>
+      <c r="D61" s="23"/>
+      <c r="E61" s="23"/>
+      <c r="F61" s="23"/>
+      <c r="G61" s="23"/>
+      <c r="H61" s="22"/>
     </row>
     <row r="62" ht="16" customHeight="1" spans="1:8">
-      <c r="A62" s="22"/>
-      <c r="B62" s="22"/>
-      <c r="C62" s="22"/>
-      <c r="D62" s="22"/>
-      <c r="E62" s="22"/>
-      <c r="F62" s="22"/>
-      <c r="G62" s="22"/>
-      <c r="H62" s="21"/>
+      <c r="A62" s="23"/>
+      <c r="B62" s="23"/>
+      <c r="C62" s="23"/>
+      <c r="D62" s="23"/>
+      <c r="E62" s="23"/>
+      <c r="F62" s="23"/>
+      <c r="G62" s="23"/>
+      <c r="H62" s="22"/>
     </row>
     <row r="63" ht="16" customHeight="1" spans="1:8">
-      <c r="A63" s="22"/>
-      <c r="B63" s="22"/>
-      <c r="C63" s="22"/>
-      <c r="D63" s="22"/>
-      <c r="E63" s="22"/>
-      <c r="F63" s="22"/>
-      <c r="G63" s="22"/>
-      <c r="H63" s="21"/>
+      <c r="A63" s="23"/>
+      <c r="B63" s="23"/>
+      <c r="C63" s="23"/>
+      <c r="D63" s="23"/>
+      <c r="E63" s="23"/>
+      <c r="F63" s="23"/>
+      <c r="G63" s="23"/>
+      <c r="H63" s="22"/>
     </row>
     <row r="64" ht="16" customHeight="1" spans="1:8">
-      <c r="A64" s="22"/>
-      <c r="B64" s="22"/>
-      <c r="C64" s="22"/>
-      <c r="D64" s="22"/>
-      <c r="E64" s="22"/>
-      <c r="F64" s="22"/>
-      <c r="G64" s="22"/>
-      <c r="H64" s="21"/>
+      <c r="A64" s="23"/>
+      <c r="B64" s="23"/>
+      <c r="C64" s="23"/>
+      <c r="D64" s="23"/>
+      <c r="E64" s="23"/>
+      <c r="F64" s="23"/>
+      <c r="G64" s="23"/>
+      <c r="H64" s="22"/>
     </row>
     <row r="65" ht="16" customHeight="1" spans="1:8">
-      <c r="A65" s="22"/>
-      <c r="B65" s="22"/>
-      <c r="C65" s="22"/>
-      <c r="D65" s="22"/>
-      <c r="E65" s="22"/>
-      <c r="F65" s="22"/>
-      <c r="G65" s="22"/>
-      <c r="H65" s="21"/>
+      <c r="A65" s="23"/>
+      <c r="B65" s="23"/>
+      <c r="C65" s="23"/>
+      <c r="D65" s="23"/>
+      <c r="E65" s="23"/>
+      <c r="F65" s="23"/>
+      <c r="G65" s="23"/>
+      <c r="H65" s="22"/>
     </row>
     <row r="66" ht="16" customHeight="1" spans="1:8">
-      <c r="A66" s="22"/>
-      <c r="B66" s="22"/>
-      <c r="C66" s="22"/>
-      <c r="D66" s="22"/>
-      <c r="E66" s="22"/>
-      <c r="F66" s="22"/>
-      <c r="G66" s="22"/>
-      <c r="H66" s="21"/>
+      <c r="A66" s="23"/>
+      <c r="B66" s="23"/>
+      <c r="C66" s="23"/>
+      <c r="D66" s="23"/>
+      <c r="E66" s="23"/>
+      <c r="F66" s="23"/>
+      <c r="G66" s="23"/>
+      <c r="H66" s="22"/>
     </row>
     <row r="67" ht="16" customHeight="1" spans="1:8">
-      <c r="A67" s="22"/>
-      <c r="B67" s="22"/>
-      <c r="C67" s="22"/>
-      <c r="D67" s="22"/>
-      <c r="E67" s="22"/>
-      <c r="F67" s="22"/>
-      <c r="G67" s="22"/>
-      <c r="H67" s="21"/>
+      <c r="A67" s="23"/>
+      <c r="B67" s="23"/>
+      <c r="C67" s="23"/>
+      <c r="D67" s="23"/>
+      <c r="E67" s="23"/>
+      <c r="F67" s="23"/>
+      <c r="G67" s="23"/>
+      <c r="H67" s="22"/>
     </row>
     <row r="68" ht="16" customHeight="1" spans="1:8">
-      <c r="A68" s="22"/>
-      <c r="B68" s="22"/>
-      <c r="C68" s="22"/>
-      <c r="D68" s="22"/>
-      <c r="E68" s="22"/>
-      <c r="F68" s="22"/>
-      <c r="G68" s="22"/>
-      <c r="H68" s="21"/>
+      <c r="A68" s="23"/>
+      <c r="B68" s="23"/>
+      <c r="C68" s="23"/>
+      <c r="D68" s="23"/>
+      <c r="E68" s="23"/>
+      <c r="F68" s="23"/>
+      <c r="G68" s="23"/>
+      <c r="H68" s="22"/>
     </row>
     <row r="69" spans="1:7">
       <c r="A69" s="3"/>
@@ -4296,7 +4311,7 @@
       <c r="D72" s="9"/>
     </row>
     <row r="73" spans="1:3">
-      <c r="A73" s="24" t="s">
+      <c r="A73" s="25" t="s">
         <v>113</v>
       </c>
       <c r="B73" s="9"/>
@@ -4305,7 +4320,7 @@
       </c>
     </row>
     <row r="74" spans="1:1">
-      <c r="A74" s="25" t="s">
+      <c r="A74" s="26" t="s">
         <v>115</v>
       </c>
     </row>
@@ -4355,7 +4370,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="13" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -4369,25 +4384,25 @@
       <c r="C3" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G3" s="11"/>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" spans="3:7">
       <c r="C4" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G4" s="11"/>
+      <c r="G4" s="13"/>
     </row>
     <row r="5" spans="4:7">
       <c r="D5" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="G5" s="11"/>
+      <c r="G5" s="13"/>
     </row>
     <row r="6" spans="4:7">
       <c r="D6" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="G6" s="11"/>
+      <c r="G6" s="13"/>
     </row>
     <row r="7" spans="3:3">
       <c r="C7" s="1" t="s">
@@ -4438,7 +4453,7 @@
       </c>
     </row>
     <row r="16" ht="14.5" spans="2:4">
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="17" t="s">
         <v>129</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -4446,43 +4461,43 @@
       </c>
     </row>
     <row r="17" ht="14.5" spans="2:5">
-      <c r="B17" s="16"/>
+      <c r="B17" s="17"/>
       <c r="C17" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="13" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="18" ht="14.5" spans="2:4">
-      <c r="B18" s="16"/>
+      <c r="B18" s="17"/>
       <c r="D18" s="1" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="19" ht="14.5" spans="2:2">
-      <c r="B19" s="16"/>
+      <c r="B19" s="17"/>
     </row>
     <row r="20" ht="14.5" spans="1:3">
       <c r="A20" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B20" s="16"/>
+      <c r="B20" s="17"/>
       <c r="C20" s="1" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="21" ht="14.5" spans="2:2">
-      <c r="B21" s="16"/>
+      <c r="B21" s="17"/>
     </row>
     <row r="22" ht="14.5" spans="2:3">
-      <c r="B22" s="16"/>
+      <c r="B22" s="17"/>
       <c r="C22" s="1" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="23" ht="14.5" spans="2:4">
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="17" t="s">
         <v>135</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -4490,19 +4505,19 @@
       </c>
     </row>
     <row r="24" ht="14.5" spans="2:3">
-      <c r="B24" s="16"/>
+      <c r="B24" s="17"/>
       <c r="C24" s="1" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="25" ht="14.5" spans="2:2">
-      <c r="B25" s="16"/>
+      <c r="B25" s="17"/>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="18" t="s">
         <v>138</v>
       </c>
     </row>
@@ -4811,76 +4826,76 @@
       <c r="C73" s="9"/>
     </row>
     <row r="74" spans="1:6">
-      <c r="A74" s="18"/>
-      <c r="B74" s="18"/>
-      <c r="C74" s="18"/>
-      <c r="D74" s="18"/>
-      <c r="E74" s="18"/>
-      <c r="F74" s="18"/>
+      <c r="A74" s="19"/>
+      <c r="B74" s="19"/>
+      <c r="C74" s="19"/>
+      <c r="D74" s="19"/>
+      <c r="E74" s="19"/>
+      <c r="F74" s="19"/>
     </row>
     <row r="75" spans="1:6">
-      <c r="A75" s="18"/>
-      <c r="B75" s="18"/>
-      <c r="C75" s="18"/>
-      <c r="D75" s="18"/>
-      <c r="E75" s="18"/>
-      <c r="F75" s="18"/>
+      <c r="A75" s="19"/>
+      <c r="B75" s="19"/>
+      <c r="C75" s="19"/>
+      <c r="D75" s="19"/>
+      <c r="E75" s="19"/>
+      <c r="F75" s="19"/>
     </row>
     <row r="76" spans="1:6">
-      <c r="A76" s="18"/>
-      <c r="B76" s="18"/>
-      <c r="C76" s="18"/>
-      <c r="D76" s="18"/>
-      <c r="E76" s="18"/>
-      <c r="F76" s="18"/>
+      <c r="A76" s="19"/>
+      <c r="B76" s="19"/>
+      <c r="C76" s="19"/>
+      <c r="D76" s="19"/>
+      <c r="E76" s="19"/>
+      <c r="F76" s="19"/>
     </row>
     <row r="77" spans="1:6">
-      <c r="A77" s="18"/>
-      <c r="B77" s="18"/>
-      <c r="C77" s="18"/>
-      <c r="D77" s="18"/>
-      <c r="E77" s="18"/>
-      <c r="F77" s="18"/>
+      <c r="A77" s="19"/>
+      <c r="B77" s="19"/>
+      <c r="C77" s="19"/>
+      <c r="D77" s="19"/>
+      <c r="E77" s="19"/>
+      <c r="F77" s="19"/>
     </row>
     <row r="78" spans="1:6">
-      <c r="A78" s="18"/>
-      <c r="B78" s="18"/>
-      <c r="C78" s="18"/>
-      <c r="D78" s="18"/>
-      <c r="E78" s="18"/>
-      <c r="F78" s="18"/>
+      <c r="A78" s="19"/>
+      <c r="B78" s="19"/>
+      <c r="C78" s="19"/>
+      <c r="D78" s="19"/>
+      <c r="E78" s="19"/>
+      <c r="F78" s="19"/>
     </row>
     <row r="79" spans="1:6">
-      <c r="A79" s="18"/>
-      <c r="B79" s="18"/>
-      <c r="C79" s="18"/>
-      <c r="D79" s="18"/>
-      <c r="E79" s="18"/>
-      <c r="F79" s="18"/>
+      <c r="A79" s="19"/>
+      <c r="B79" s="19"/>
+      <c r="C79" s="19"/>
+      <c r="D79" s="19"/>
+      <c r="E79" s="19"/>
+      <c r="F79" s="19"/>
     </row>
     <row r="80" spans="1:6">
-      <c r="A80" s="18"/>
-      <c r="B80" s="18"/>
-      <c r="C80" s="18"/>
-      <c r="D80" s="18"/>
-      <c r="E80" s="18"/>
-      <c r="F80" s="18"/>
+      <c r="A80" s="19"/>
+      <c r="B80" s="19"/>
+      <c r="C80" s="19"/>
+      <c r="D80" s="19"/>
+      <c r="E80" s="19"/>
+      <c r="F80" s="19"/>
     </row>
     <row r="81" spans="1:6">
-      <c r="A81" s="18"/>
-      <c r="B81" s="18"/>
-      <c r="C81" s="18"/>
-      <c r="D81" s="18"/>
-      <c r="E81" s="18"/>
-      <c r="F81" s="18"/>
+      <c r="A81" s="19"/>
+      <c r="B81" s="19"/>
+      <c r="C81" s="19"/>
+      <c r="D81" s="19"/>
+      <c r="E81" s="19"/>
+      <c r="F81" s="19"/>
     </row>
     <row r="82" spans="1:6">
-      <c r="A82" s="18"/>
-      <c r="B82" s="18"/>
-      <c r="C82" s="18"/>
-      <c r="D82" s="18"/>
-      <c r="E82" s="18"/>
-      <c r="F82" s="18"/>
+      <c r="A82" s="19"/>
+      <c r="B82" s="19"/>
+      <c r="C82" s="19"/>
+      <c r="D82" s="19"/>
+      <c r="E82" s="19"/>
+      <c r="F82" s="19"/>
     </row>
     <row r="93" spans="3:4">
       <c r="C93" s="9"/>
@@ -4933,7 +4948,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="7:7">
-      <c r="G1" s="11"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
@@ -4948,7 +4963,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="13" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -5001,7 +5016,7 @@
     <col min="4" max="4" width="3.33076923076923" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.6692307692308" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.1692307692308" style="1" customWidth="1"/>
-    <col min="7" max="7" width="4.5" style="15" customWidth="1"/>
+    <col min="7" max="7" width="4.5" style="16" customWidth="1"/>
     <col min="8" max="8" width="4.5" style="1" customWidth="1"/>
     <col min="9" max="16384" width="8.66923076923077" style="1"/>
   </cols>
@@ -5024,7 +5039,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="13" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -5304,7 +5319,7 @@
       <c r="D36" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="G36" s="15">
+      <c r="G36" s="16">
         <v>5</v>
       </c>
     </row>
@@ -5360,36 +5375,36 @@
   <dimension ref="A1:H94"/>
   <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="14" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="25.4153846153846" style="12" customWidth="1"/>
-    <col min="2" max="2" width="19.8307692307692" style="12" customWidth="1"/>
-    <col min="3" max="3" width="5.66923076923077" style="12" customWidth="1"/>
-    <col min="4" max="4" width="7.08461538461538" style="12" customWidth="1"/>
-    <col min="5" max="5" width="7.75384615384615" style="12" customWidth="1"/>
-    <col min="6" max="6" width="12.1692307692308" style="12" customWidth="1"/>
-    <col min="7" max="7" width="4.5" style="13" customWidth="1"/>
-    <col min="8" max="8" width="4.5" style="12" customWidth="1"/>
-    <col min="9" max="16384" width="8.66923076923077" style="12"/>
+    <col min="1" max="1" width="25.4153846153846" style="11" customWidth="1"/>
+    <col min="2" max="2" width="19.8307692307692" style="11" customWidth="1"/>
+    <col min="3" max="3" width="5.66923076923077" style="11" customWidth="1"/>
+    <col min="4" max="4" width="7.08461538461538" style="11" customWidth="1"/>
+    <col min="5" max="5" width="7.75384615384615" style="11" customWidth="1"/>
+    <col min="6" max="6" width="12.1692307692308" style="11" customWidth="1"/>
+    <col min="7" max="7" width="4.5" style="14" customWidth="1"/>
+    <col min="8" max="8" width="4.5" style="11" customWidth="1"/>
+    <col min="9" max="16384" width="8.66923076923077" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2">
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="2" spans="2:8">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="11" t="s">
         <v>6</v>
       </c>
     </row>
@@ -5409,21 +5424,21 @@
     </row>
     <row r="5" spans="3:5">
       <c r="C5" s="10"/>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="11" t="s">
         <v>256</v>
       </c>
       <c r="E5" s="10"/>
     </row>
     <row r="6" spans="3:5">
       <c r="C6" s="10"/>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="11" t="s">
         <v>257</v>
       </c>
       <c r="E6" s="10"/>
     </row>
     <row r="7" spans="3:5">
       <c r="C7" s="10"/>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="11" t="s">
         <v>258</v>
       </c>
       <c r="E7" s="10"/>
@@ -5436,7 +5451,7 @@
       <c r="E8" s="10"/>
     </row>
     <row r="9" spans="4:4">
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="11" t="s">
         <v>260</v>
       </c>
     </row>
@@ -5478,127 +5493,127 @@
       <c r="D18" s="1"/>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="11" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="20" spans="2:3">
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="11" t="s">
         <v>267</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="11" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="21" spans="1:3">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="11" t="s">
         <v>269</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="11" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="11" t="s">
         <v>271</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D22" s="11" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="23" spans="4:4">
-      <c r="D23" s="12" t="s">
+      <c r="D23" s="11" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="24" spans="4:4">
-      <c r="D24" s="12" t="s">
+      <c r="D24" s="11" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="25" spans="4:4">
-      <c r="D25" s="12" t="s">
+      <c r="D25" s="11" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="11" t="s">
         <v>276</v>
       </c>
-      <c r="E26" s="12" t="s">
+      <c r="E26" s="11" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="11" t="s">
         <v>278</v>
       </c>
-      <c r="E27" s="12" t="s">
+      <c r="E27" s="11" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="28" spans="5:5">
-      <c r="E28" s="12" t="s">
+      <c r="E28" s="11" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="29" spans="4:4">
-      <c r="D29" s="12" t="s">
+      <c r="D29" s="11" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="30" spans="1:4">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="11" t="s">
         <v>282</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="11" t="s">
         <v>283</v>
       </c>
-      <c r="D30" s="12" t="s">
+      <c r="D30" s="11" t="s">
         <v>284</v>
       </c>
     </row>
     <row r="31" spans="3:3">
-      <c r="C31" s="12" t="s">
+      <c r="C31" s="11" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="11" t="s">
         <v>286</v>
       </c>
-      <c r="D32" s="12" t="s">
+      <c r="D32" s="11" t="s">
         <v>287</v>
       </c>
-      <c r="E32" s="12" t="s">
+      <c r="E32" s="11" t="s">
         <v>288</v>
       </c>
-      <c r="F32" s="12" t="s">
+      <c r="F32" s="11" t="s">
         <v>289</v>
       </c>
     </row>
     <row r="33" spans="4:5">
-      <c r="D33" s="12" t="s">
+      <c r="D33" s="11" t="s">
         <v>290</v>
       </c>
-      <c r="E33" s="12" t="s">
+      <c r="E33" s="11" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="34" spans="1:6">
-      <c r="A34" s="12" t="s">
+      <c r="A34" s="11" t="s">
         <v>292</v>
       </c>
-      <c r="B34" s="12" t="s">
+      <c r="B34" s="11" t="s">
         <v>293</v>
       </c>
-      <c r="D34" s="12" t="s">
+      <c r="D34" s="11" t="s">
         <v>294</v>
       </c>
-      <c r="F34" s="12" t="s">
+      <c r="F34" s="11" t="s">
         <v>295</v>
       </c>
     </row>
@@ -5643,305 +5658,305 @@
       </c>
     </row>
     <row r="43" spans="3:3">
-      <c r="C43" s="12" t="s">
+      <c r="C43" s="11" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="44" spans="4:5">
-      <c r="D44" s="12" t="s">
+      <c r="D44" s="11" t="s">
         <v>303</v>
       </c>
-      <c r="E44" s="12" t="s">
+      <c r="E44" s="11" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="45" spans="5:5">
-      <c r="E45" s="12" t="s">
+      <c r="E45" s="11" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="47" spans="4:4">
-      <c r="D47" s="12" t="s">
+      <c r="D47" s="11" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="48" spans="5:5">
-      <c r="E48" s="12" t="s">
+      <c r="E48" s="11" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="49" spans="5:5">
-      <c r="E49" s="12" t="s">
+      <c r="E49" s="11" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="50" spans="5:5">
-      <c r="E50" s="12" t="s">
+      <c r="E50" s="11" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="51" spans="1:4">
-      <c r="A51" s="12" t="s">
+      <c r="A51" s="11" t="s">
         <v>310</v>
       </c>
-      <c r="D51" s="12" t="s">
+      <c r="D51" s="11" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="52" spans="3:3">
-      <c r="C52" s="12" t="s">
+      <c r="C52" s="11" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="53" spans="4:5">
-      <c r="D53" s="12" t="s">
+      <c r="D53" s="11" t="s">
         <v>313</v>
       </c>
-      <c r="E53" s="12" t="s">
+      <c r="E53" s="11" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="54" spans="5:5">
-      <c r="E54" s="12" t="s">
+      <c r="E54" s="11" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="55" spans="4:4">
-      <c r="D55" s="12" t="s">
+      <c r="D55" s="11" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="56" spans="1:3">
-      <c r="A56" s="12" t="s">
+      <c r="A56" s="11" t="s">
         <v>317</v>
       </c>
-      <c r="B56" s="12" t="s">
+      <c r="B56" s="11" t="s">
         <v>318</v>
       </c>
-      <c r="C56" s="12" t="s">
+      <c r="C56" s="11" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="57" spans="2:4">
-      <c r="B57" s="12" t="s">
+      <c r="B57" s="11" t="s">
         <v>320</v>
       </c>
-      <c r="D57" s="12" t="s">
+      <c r="D57" s="11" t="s">
         <v>321</v>
       </c>
     </row>
     <row r="58" spans="1:2">
-      <c r="A58" s="12" t="s">
+      <c r="A58" s="11" t="s">
         <v>322</v>
       </c>
-      <c r="B58" s="12" t="s">
+      <c r="B58" s="11" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="59" spans="3:3">
-      <c r="C59" s="12" t="s">
+      <c r="C59" s="11" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="60" spans="4:4">
-      <c r="D60" s="12" t="s">
+      <c r="D60" s="11" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="61" spans="3:3">
-      <c r="C61" s="12" t="s">
+      <c r="C61" s="11" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="62" spans="2:4">
-      <c r="B62" s="12" t="s">
+      <c r="B62" s="11" t="s">
         <v>327</v>
       </c>
-      <c r="D62" s="12" t="s">
+      <c r="D62" s="11" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="63" spans="2:2">
-      <c r="B63" s="12" t="s">
+      <c r="B63" s="11" t="s">
         <v>329</v>
       </c>
     </row>
     <row r="64" spans="3:3">
-      <c r="C64" s="12" t="s">
+      <c r="C64" s="11" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="65" spans="4:5">
-      <c r="D65" s="12" t="s">
+      <c r="D65" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="E65" s="12" t="s">
+      <c r="E65" s="11" t="s">
         <v>332</v>
       </c>
     </row>
     <row r="66" spans="1:4">
-      <c r="A66" s="12" t="s">
+      <c r="A66" s="11" t="s">
         <v>333</v>
       </c>
-      <c r="D66" s="12" t="s">
+      <c r="D66" s="11" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="67" spans="1:4">
-      <c r="A67" s="12" t="s">
+      <c r="A67" s="11" t="s">
         <v>335</v>
       </c>
-      <c r="B67" s="12" t="s">
+      <c r="B67" s="11" t="s">
         <v>336</v>
       </c>
-      <c r="D67" s="12" t="s">
+      <c r="D67" s="11" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="68" spans="2:2">
-      <c r="B68" s="12" t="s">
+      <c r="B68" s="11" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="69" spans="2:2">
-      <c r="B69" s="12" t="s">
+      <c r="B69" s="11" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="71" spans="3:3">
-      <c r="C71" s="12" t="s">
+      <c r="C71" s="11" t="s">
         <v>340</v>
       </c>
     </row>
     <row r="72" spans="4:4">
-      <c r="D72" s="12" t="s">
+      <c r="D72" s="11" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="73" spans="4:4">
-      <c r="D73" s="12" t="s">
+      <c r="D73" s="11" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="74" spans="4:4">
-      <c r="D74" s="12" t="s">
+      <c r="D74" s="11" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="75" spans="4:4">
-      <c r="D75" s="12" t="s">
+      <c r="D75" s="11" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="76" spans="1:3">
-      <c r="A76" s="12" t="s">
+      <c r="A76" s="11" t="s">
         <v>345</v>
       </c>
-      <c r="C76" s="12" t="s">
+      <c r="C76" s="11" t="s">
         <v>346</v>
       </c>
     </row>
     <row r="77" spans="2:4">
-      <c r="B77" s="12" t="s">
+      <c r="B77" s="11" t="s">
         <v>347</v>
       </c>
-      <c r="D77" s="12" t="s">
+      <c r="D77" s="11" t="s">
         <v>348</v>
       </c>
     </row>
     <row r="78" spans="1:3">
-      <c r="A78" s="12" t="s">
+      <c r="A78" s="11" t="s">
         <v>349</v>
       </c>
-      <c r="C78" s="12" t="s">
+      <c r="C78" s="11" t="s">
         <v>350</v>
       </c>
     </row>
     <row r="79" spans="4:4">
-      <c r="D79" s="12" t="s">
+      <c r="D79" s="11" t="s">
         <v>351</v>
       </c>
     </row>
     <row r="80" spans="2:3">
-      <c r="B80" s="12" t="s">
+      <c r="B80" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="C80" s="12" t="s">
+      <c r="C80" s="11" t="s">
         <v>353</v>
       </c>
     </row>
     <row r="81" spans="3:3">
-      <c r="C81" s="12" t="s">
+      <c r="C81" s="11" t="s">
         <v>354</v>
       </c>
     </row>
     <row r="82" spans="1:3">
-      <c r="A82" s="12" t="s">
+      <c r="A82" s="11" t="s">
         <v>355</v>
       </c>
-      <c r="C82" s="12" t="s">
+      <c r="C82" s="11" t="s">
         <v>356</v>
       </c>
     </row>
     <row r="83" spans="4:4">
-      <c r="D83" s="12" t="s">
+      <c r="D83" s="11" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="84" spans="4:4">
-      <c r="D84" s="12" t="s">
+      <c r="D84" s="11" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="85" spans="1:3">
-      <c r="A85" s="12" t="s">
+      <c r="A85" s="11" t="s">
         <v>359</v>
       </c>
-      <c r="C85" s="12" t="s">
+      <c r="C85" s="11" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="86" spans="3:3">
-      <c r="C86" s="12" t="s">
+      <c r="C86" s="11" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="87" spans="4:4">
-      <c r="D87" s="12" t="s">
+      <c r="D87" s="11" t="s">
         <v>362</v>
       </c>
     </row>
     <row r="88" spans="4:4">
-      <c r="D88" s="12" t="s">
+      <c r="D88" s="11" t="s">
         <v>363</v>
       </c>
     </row>
     <row r="91" spans="1:3">
-      <c r="A91" s="12" t="s">
+      <c r="A91" s="11" t="s">
         <v>364</v>
       </c>
-      <c r="C91" s="12" t="s">
+      <c r="C91" s="11" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="92" spans="4:4">
-      <c r="D92" s="12" t="s">
+      <c r="D92" s="11" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="93" spans="4:4">
-      <c r="D93" s="12" t="s">
+      <c r="D93" s="11" t="s">
         <v>367</v>
       </c>
     </row>
     <row r="94" spans="1:7">
-      <c r="A94" s="12" t="s">
+      <c r="A94" s="11" t="s">
         <v>368</v>
       </c>
-      <c r="C94" s="12" t="s">
+      <c r="C94" s="11" t="s">
         <v>369</v>
       </c>
-      <c r="G94" s="13">
+      <c r="G94" s="14">
         <v>5</v>
       </c>
     </row>
@@ -5981,7 +5996,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="13" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -6049,7 +6064,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A3:D42"/>
+  <dimension ref="A3:D46"/>
   <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="12.5" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="8.66923076923077" style="8"/>
@@ -6382,6 +6397,23 @@
       </c>
       <c r="D42" s="10"/>
     </row>
+    <row r="43" ht="15.5"/>
+    <row r="44" ht="14" spans="2:3">
+      <c r="B44" s="11" t="s">
+        <v>436</v>
+      </c>
+      <c r="C44" s="11" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="46" ht="14" spans="2:3">
+      <c r="B46" s="12" t="s">
+        <v>438</v>
+      </c>
+      <c r="C46" s="11" t="s">
+        <v>439</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
improved topic list for pandas
</commit_message>
<xml_diff>
--- a/p/py-25/py-core/topic-list_py.xlsx
+++ b/p/py-25/py-core/topic-list_py.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12200" tabRatio="698" firstSheet="1" activeTab="8"/>
+    <workbookView windowWidth="28800" windowHeight="12200" tabRatio="698" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="core" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="501">
   <si>
     <t>Most basic things in py</t>
   </si>
@@ -368,6 +368,21 @@
     <t>for in filter, for in compress, for in groupby</t>
   </si>
   <si>
+    <t>garbage collector</t>
+  </si>
+  <si>
+    <t>gc.collect()</t>
+  </si>
+  <si>
+    <t>import gc</t>
+  </si>
+  <si>
+    <t>datacamp.com/tutorial/python-garbage-collection</t>
+  </si>
+  <si>
+    <t>weakref</t>
+  </si>
+  <si>
     <t>py debuggers</t>
   </si>
   <si>
@@ -462,6 +477,9 @@
   </si>
   <si>
     <t>Basics 804 Set</t>
+  </si>
+  <si>
+    <t>isdigit90</t>
   </si>
   <si>
     <t>bitwise operators</t>
@@ -3277,12 +3295,12 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="2" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
     </row>
     <row r="3" spans="1:1">
@@ -3290,7 +3308,7 @@
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="4" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
     </row>
     <row r="5" spans="1:1">
@@ -3298,32 +3316,32 @@
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="5" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="5" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="6" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="6" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="6" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="5" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
     </row>
     <row r="12" spans="1:1">
@@ -3331,7 +3349,7 @@
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="4" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
     </row>
     <row r="14" spans="1:1">
@@ -3339,32 +3357,32 @@
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="5" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="5" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="6" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="6" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="6" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="5" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
     </row>
     <row r="21" spans="1:1">
@@ -3372,51 +3390,51 @@
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="4" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="3" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="3"/>
       <c r="B24" s="1" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" s="5" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" s="5" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" s="6" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" s="6" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" s="6" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" s="5" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
     </row>
     <row r="31" spans="1:1">
@@ -3424,7 +3442,7 @@
     </row>
     <row r="32" spans="1:1">
       <c r="A32" s="4" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
     </row>
     <row r="33" spans="1:1">
@@ -3432,32 +3450,32 @@
     </row>
     <row r="34" spans="1:1">
       <c r="A34" s="5" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" s="5" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" s="6" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" s="6" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" s="6" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" s="5" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
     </row>
     <row r="40" spans="1:1">
@@ -3465,7 +3483,7 @@
     </row>
     <row r="41" spans="1:1">
       <c r="A41" s="4" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
     </row>
     <row r="42" spans="1:1">
@@ -3473,32 +3491,32 @@
     </row>
     <row r="43" spans="1:1">
       <c r="A43" s="5" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" s="5" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" s="6" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" s="6" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" s="6" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" s="5" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
     </row>
     <row r="49" spans="1:1">
@@ -3506,7 +3524,7 @@
     </row>
     <row r="50" spans="1:1">
       <c r="A50" s="4" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
     </row>
     <row r="51" spans="1:1">
@@ -3514,32 +3532,32 @@
     </row>
     <row r="52" spans="1:1">
       <c r="A52" s="5" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
     </row>
     <row r="53" spans="1:1">
       <c r="A53" s="5" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" s="6" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
     </row>
     <row r="55" spans="1:1">
       <c r="A55" s="6" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
     </row>
     <row r="56" spans="1:1">
       <c r="A56" s="6" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
     </row>
     <row r="57" spans="1:1">
       <c r="A57" s="5" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
     </row>
     <row r="58" spans="1:1">
@@ -3547,7 +3565,7 @@
     </row>
     <row r="59" spans="1:1">
       <c r="A59" s="4" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
     </row>
     <row r="60" spans="1:1">
@@ -3555,32 +3573,32 @@
     </row>
     <row r="61" spans="1:1">
       <c r="A61" s="5" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
     </row>
     <row r="62" spans="1:1">
       <c r="A62" s="5" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
     </row>
     <row r="63" spans="1:1">
       <c r="A63" s="6" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
     </row>
     <row r="64" spans="1:1">
       <c r="A64" s="6" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
     </row>
     <row r="65" spans="1:1">
       <c r="A65" s="6" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
     </row>
     <row r="66" spans="1:1">
       <c r="A66" s="5" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
     </row>
     <row r="67" spans="1:1">
@@ -3588,37 +3606,37 @@
     </row>
     <row r="68" spans="1:1">
       <c r="A68" s="4" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
     </row>
     <row r="69" spans="1:1">
       <c r="A69" s="2" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
     </row>
     <row r="70" spans="1:1">
       <c r="A70" s="1" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
     </row>
     <row r="71" spans="1:1">
       <c r="A71" s="1" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
     </row>
     <row r="73" spans="1:1">
       <c r="A73" s="7" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
     </row>
     <row r="74" spans="1:1">
       <c r="A74" s="1" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
     </row>
     <row r="75" spans="1:1">
       <c r="A75" s="1" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -4046,7 +4064,9 @@
     <row r="46" ht="16" customHeight="1" spans="1:8">
       <c r="A46" s="23"/>
       <c r="B46" s="23"/>
-      <c r="C46" s="23"/>
+      <c r="C46" s="23" t="s">
+        <v>110</v>
+      </c>
       <c r="D46" s="23"/>
       <c r="E46" s="23"/>
       <c r="F46" s="23"/>
@@ -4055,18 +4075,26 @@
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:8">
       <c r="A47" s="23"/>
-      <c r="B47" s="23"/>
+      <c r="B47" s="23" t="s">
+        <v>111</v>
+      </c>
       <c r="C47" s="23"/>
-      <c r="D47" s="23"/>
+      <c r="D47" s="23" t="s">
+        <v>112</v>
+      </c>
       <c r="E47" s="23"/>
       <c r="F47" s="23"/>
       <c r="G47" s="23"/>
       <c r="H47" s="22"/>
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:8">
-      <c r="A48" s="23"/>
+      <c r="A48" s="23" t="s">
+        <v>113</v>
+      </c>
       <c r="B48" s="23"/>
-      <c r="C48" s="23"/>
+      <c r="C48" s="23" t="s">
+        <v>114</v>
+      </c>
       <c r="D48" s="23"/>
       <c r="E48" s="23"/>
       <c r="F48" s="23"/>
@@ -4277,7 +4305,7 @@
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="9" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D69" s="9"/>
       <c r="E69" s="3"/>
@@ -4288,7 +4316,7 @@
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="9" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="D70" s="9"/>
       <c r="E70" s="3"/>
@@ -4300,7 +4328,7 @@
       <c r="B71" s="3"/>
       <c r="C71" s="9"/>
       <c r="D71" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
@@ -4312,16 +4340,16 @@
     </row>
     <row r="73" spans="1:3">
       <c r="A73" s="25" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B73" s="9"/>
       <c r="C73" s="9" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="74" spans="1:1">
       <c r="A74" s="26" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -4354,7 +4382,7 @@
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" s="1" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -4379,100 +4407,100 @@
     </row>
     <row r="3" spans="2:7">
       <c r="B3" s="1" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="G3" s="13"/>
     </row>
     <row r="4" spans="3:7">
       <c r="C4" s="1" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="G4" s="13"/>
     </row>
     <row r="5" spans="4:7">
       <c r="D5" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="G5" s="13"/>
     </row>
     <row r="6" spans="4:7">
       <c r="D6" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="G6" s="13"/>
     </row>
     <row r="7" spans="3:3">
       <c r="C7" s="1" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="4:4">
       <c r="D8" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="5:5">
       <c r="E9" s="1" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="4:4">
       <c r="D10" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="4:4">
       <c r="D11" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="5:5">
       <c r="E12" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="3:3">
       <c r="C14" s="1" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="4:4">
       <c r="D15" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" ht="14.5" spans="2:4">
       <c r="B16" s="17" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" ht="14.5" spans="2:5">
       <c r="B17" s="17"/>
       <c r="C17" s="1" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18" ht="14.5" spans="2:4">
       <c r="B18" s="17"/>
       <c r="D18" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" ht="14.5" spans="2:2">
@@ -4480,11 +4508,11 @@
     </row>
     <row r="20" ht="14.5" spans="1:3">
       <c r="A20" s="1" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="1" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="21" ht="14.5" spans="2:2">
@@ -4493,21 +4521,21 @@
     <row r="22" ht="14.5" spans="2:3">
       <c r="B22" s="17"/>
       <c r="C22" s="1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" ht="14.5" spans="2:4">
       <c r="B23" s="17" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" ht="14.5" spans="2:3">
       <c r="B24" s="17"/>
       <c r="C24" s="1" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" ht="14.5" spans="2:2">
@@ -4515,311 +4543,314 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="27" spans="3:5">
       <c r="C27" s="1" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="1" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="4:4">
+    <row r="29" spans="2:4">
+      <c r="B29" s="1" t="s">
+        <v>147</v>
+      </c>
       <c r="D29" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="4:4">
       <c r="D30" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="31" spans="4:4">
       <c r="D31" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="32" spans="4:4">
       <c r="D32" s="1" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="1" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="34" spans="3:3">
       <c r="C34" s="1" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="35" spans="3:3">
       <c r="C35" s="1" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="36" spans="4:4">
       <c r="D36" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="37" spans="2:5">
       <c r="B37" s="1" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
     <row r="38" spans="2:6">
       <c r="B38" s="1" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="1" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="40" spans="2:4">
       <c r="B40" s="1" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="1" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="42" spans="2:2">
       <c r="B42" s="1" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="1" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="44" spans="2:2">
       <c r="B44" s="1" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
     </row>
     <row r="45" spans="4:4">
       <c r="D45" s="1" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="46" spans="5:5">
       <c r="E46" s="1" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="1" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
     </row>
     <row r="48" spans="2:4">
       <c r="B48" s="1" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="49" spans="4:4">
       <c r="D49" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="50" spans="3:3">
       <c r="C50" s="1" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
     </row>
     <row r="51" spans="4:4">
       <c r="D51" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="1" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
     </row>
     <row r="53" spans="5:5">
       <c r="E53" s="1" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
     </row>
     <row r="55" spans="4:4">
       <c r="D55" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="56" spans="4:4">
       <c r="D56" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="1" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="1" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="59" spans="2:2">
       <c r="B59" s="1" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="1" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="61" spans="2:2">
       <c r="B61" s="1" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="62" spans="3:3">
       <c r="C62" s="1" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="63" spans="4:4">
       <c r="D63" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="64" spans="4:4">
       <c r="D64" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="65" spans="4:4">
       <c r="D65" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="67" spans="3:3">
       <c r="C67" s="9" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
     </row>
     <row r="68" spans="3:4">
       <c r="C68" s="9"/>
       <c r="D68" s="9" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="69" spans="3:5">
       <c r="C69" s="9"/>
       <c r="E69" s="1" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="70" spans="3:4">
       <c r="C70" s="9"/>
       <c r="D70" s="1" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
     </row>
     <row r="71" spans="3:5">
       <c r="C71" s="9"/>
       <c r="E71" s="1" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="72" spans="3:4">
       <c r="C72" s="9"/>
       <c r="D72" s="1" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
     </row>
     <row r="73" spans="3:3">
@@ -4972,29 +5003,29 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="2:4">
       <c r="B4" s="1" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="2:5">
       <c r="B5" s="1" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -5023,7 +5054,7 @@
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" s="1" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -5048,91 +5079,91 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="2:2">
       <c r="B4" s="1" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="2:2">
       <c r="B5" s="1" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" spans="4:4">
       <c r="D9" s="1" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" spans="4:4">
       <c r="D11" s="1" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
     </row>
     <row r="12" spans="5:5">
       <c r="E12" s="1" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13" spans="3:3">
       <c r="C13" s="1" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" spans="2:4">
       <c r="B14" s="1" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>34</v>
@@ -5140,14 +5171,14 @@
     </row>
     <row r="16" spans="4:4">
       <c r="D16" s="1" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
@@ -5158,19 +5189,19 @@
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="9" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
@@ -5181,33 +5212,33 @@
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="9" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="F23" s="9"/>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="9" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="F24" s="9"/>
     </row>
@@ -5216,29 +5247,29 @@
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="9" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="9" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
@@ -5247,10 +5278,10 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="9" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
@@ -5301,23 +5332,23 @@
     </row>
     <row r="34" spans="1:9">
       <c r="A34" s="1" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="H34" s="10"/>
       <c r="I34" s="10"/>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="1" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="G36" s="16">
         <v>5</v>
@@ -5325,42 +5356,42 @@
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="1" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="1" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
     </row>
     <row r="39" spans="5:5">
       <c r="E39" s="1" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="1" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
     </row>
     <row r="41" spans="2:2">
       <c r="B41" s="1" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -5388,7 +5419,7 @@
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" s="11" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -5410,7 +5441,7 @@
     </row>
     <row r="3" spans="3:5">
       <c r="C3" s="10" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
@@ -5418,66 +5449,66 @@
     <row r="4" spans="3:5">
       <c r="C4" s="10"/>
       <c r="D4" s="10" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="3:5">
       <c r="C5" s="10"/>
       <c r="D5" s="11" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="E5" s="10"/>
     </row>
     <row r="6" spans="3:5">
       <c r="C6" s="10"/>
       <c r="D6" s="11" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="E6" s="10"/>
     </row>
     <row r="7" spans="3:5">
       <c r="C7" s="10"/>
       <c r="D7" s="11" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="E7" s="10"/>
     </row>
     <row r="8" spans="3:5">
       <c r="C8" s="10"/>
       <c r="D8" s="10" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="E8" s="10"/>
     </row>
     <row r="9" spans="4:4">
       <c r="D9" s="11" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
     </row>
     <row r="10" spans="4:4">
       <c r="D10" s="10" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="11" spans="4:4">
       <c r="D11" s="10" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
     </row>
     <row r="12" spans="4:4">
       <c r="D12" s="1" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13" spans="4:4">
       <c r="D13" s="1" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" spans="4:4">
       <c r="D14" s="1" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="15" spans="4:4">
@@ -5494,150 +5525,150 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="11" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
     </row>
     <row r="20" spans="2:3">
       <c r="B20" s="11" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="11" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="11" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
     </row>
     <row r="23" spans="4:4">
       <c r="D23" s="11" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="24" spans="4:4">
       <c r="D24" s="11" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
     </row>
     <row r="25" spans="4:4">
       <c r="D25" s="11" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="11" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="11" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
     </row>
     <row r="28" spans="5:5">
       <c r="E28" s="11" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
     </row>
     <row r="29" spans="4:4">
       <c r="D29" s="11" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="11" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
     </row>
     <row r="31" spans="3:3">
       <c r="C31" s="11" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="11" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
     </row>
     <row r="33" spans="4:5">
       <c r="D33" s="11" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="11" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
     </row>
     <row r="35" spans="3:4">
       <c r="C35" s="10" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="D35" s="10"/>
     </row>
     <row r="36" spans="3:4">
       <c r="C36" s="10"/>
       <c r="D36" s="10" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
     </row>
     <row r="37" spans="3:4">
       <c r="C37" s="10"/>
       <c r="D37" s="10" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
     </row>
     <row r="38" spans="3:4">
       <c r="C38" s="10" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="D38" s="10"/>
     </row>
@@ -5647,314 +5678,314 @@
     </row>
     <row r="40" spans="3:4">
       <c r="C40" s="10" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="D40" s="10"/>
     </row>
     <row r="41" spans="3:4">
       <c r="C41" s="10"/>
       <c r="D41" s="10" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
     </row>
     <row r="43" spans="3:3">
       <c r="C43" s="11" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
     </row>
     <row r="44" spans="4:5">
       <c r="D44" s="11" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
     </row>
     <row r="45" spans="5:5">
       <c r="E45" s="11" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
     </row>
     <row r="47" spans="4:4">
       <c r="D47" s="11" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="48" spans="5:5">
       <c r="E48" s="11" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
     </row>
     <row r="49" spans="5:5">
       <c r="E49" s="11" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
     </row>
     <row r="50" spans="5:5">
       <c r="E50" s="11" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="11" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
     </row>
     <row r="52" spans="3:3">
       <c r="C52" s="11" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
     </row>
     <row r="53" spans="4:5">
       <c r="D53" s="11" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
     </row>
     <row r="54" spans="5:5">
       <c r="E54" s="11" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="55" spans="4:4">
       <c r="D55" s="11" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" s="11" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
     </row>
     <row r="57" spans="2:4">
       <c r="B57" s="11" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="11" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
     </row>
     <row r="59" spans="3:3">
       <c r="C59" s="11" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="60" spans="4:4">
       <c r="D60" s="11" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
     </row>
     <row r="61" spans="3:3">
       <c r="C61" s="11" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
     </row>
     <row r="62" spans="2:4">
       <c r="B62" s="11" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="D62" s="11" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
     </row>
     <row r="63" spans="2:2">
       <c r="B63" s="11" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
     </row>
     <row r="64" spans="3:3">
       <c r="C64" s="11" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
     </row>
     <row r="65" spans="4:5">
       <c r="D65" s="11" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="11" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="11" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="D67" s="11" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
     </row>
     <row r="68" spans="2:2">
       <c r="B68" s="11" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
     </row>
     <row r="69" spans="2:2">
       <c r="B69" s="11" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
     </row>
     <row r="71" spans="3:3">
       <c r="C71" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
     </row>
     <row r="72" spans="4:4">
       <c r="D72" s="11" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
     </row>
     <row r="73" spans="4:4">
       <c r="D73" s="11" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
     </row>
     <row r="74" spans="4:4">
       <c r="D74" s="11" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
     </row>
     <row r="75" spans="4:4">
       <c r="D75" s="11" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" s="11" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
     </row>
     <row r="77" spans="2:4">
       <c r="B77" s="11" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="D77" s="11" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" s="11" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="C78" s="11" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
     </row>
     <row r="79" spans="4:4">
       <c r="D79" s="11" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
     </row>
     <row r="80" spans="2:3">
       <c r="B80" s="11" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
     </row>
     <row r="81" spans="3:3">
       <c r="C81" s="11" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" s="11" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="C82" s="11" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
     </row>
     <row r="83" spans="4:4">
       <c r="D83" s="11" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
     </row>
     <row r="84" spans="4:4">
       <c r="D84" s="11" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" s="11" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="C85" s="11" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
     </row>
     <row r="86" spans="3:3">
       <c r="C86" s="11" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
     </row>
     <row r="87" spans="4:4">
       <c r="D87" s="11" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
     <row r="88" spans="4:4">
       <c r="D88" s="11" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" s="11" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="C91" s="11" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
     </row>
     <row r="92" spans="4:4">
       <c r="D92" s="11" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
     </row>
     <row r="93" spans="4:4">
       <c r="D93" s="11" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
     </row>
     <row r="94" spans="1:7">
       <c r="A94" s="11" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="C94" s="11" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="G94" s="14">
         <v>5</v>
@@ -6005,39 +6036,39 @@
     </row>
     <row r="3" spans="3:5">
       <c r="C3" s="1" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
     </row>
     <row r="4" spans="3:5">
       <c r="C4" s="1" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
     </row>
     <row r="5" spans="3:5">
       <c r="C5" s="1" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
     </row>
     <row r="6" spans="3:3">
       <c r="C6" s="1" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
     </row>
     <row r="7" spans="3:5">
       <c r="C7" s="1" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
     </row>
   </sheetData>
@@ -6075,37 +6106,37 @@
   <sheetData>
     <row r="3" spans="3:3">
       <c r="C3" s="8" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
     </row>
     <row r="5" spans="3:3">
       <c r="C5" s="8" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
     </row>
     <row r="7" spans="3:3">
       <c r="C7" s="8" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
     </row>
     <row r="8" ht="14" spans="4:4">
       <c r="D8" s="9" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
     </row>
     <row r="9" spans="3:3">
       <c r="C9" s="8" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
     </row>
     <row r="11" spans="3:3">
       <c r="C11" s="8" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
     </row>
     <row r="13" ht="14" spans="1:4">
       <c r="A13" s="10" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -6113,7 +6144,7 @@
     </row>
     <row r="14" ht="14" spans="1:4">
       <c r="A14" s="10" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -6122,50 +6153,50 @@
     <row r="15" ht="14" spans="1:4">
       <c r="A15" s="10"/>
       <c r="B15" s="10" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="D15" s="10"/>
     </row>
     <row r="16" ht="14" spans="1:4">
       <c r="A16" s="10"/>
       <c r="B16" s="10" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="D16" s="10"/>
     </row>
     <row r="17" ht="14" spans="1:4">
       <c r="A17" s="10"/>
       <c r="B17" s="10" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="D17" s="10"/>
     </row>
     <row r="18" ht="14" spans="1:4">
       <c r="A18" s="10"/>
       <c r="B18" s="10" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="D18" s="10"/>
     </row>
     <row r="19" ht="14" spans="1:4">
       <c r="A19" s="10"/>
       <c r="B19" s="10" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="D19" s="10"/>
     </row>
@@ -6173,245 +6204,244 @@
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="D20" s="10"/>
     </row>
     <row r="21" ht="14" spans="1:4">
       <c r="A21" s="10"/>
       <c r="B21" s="10" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="D21" s="10"/>
     </row>
     <row r="22" ht="14" spans="1:4">
       <c r="A22" s="10"/>
       <c r="B22" s="10" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="D22" s="10"/>
     </row>
     <row r="23" ht="14" spans="1:4">
       <c r="A23" s="10"/>
       <c r="B23" s="10" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="D23" s="10"/>
     </row>
     <row r="24" ht="14" spans="1:4">
       <c r="A24" s="10"/>
       <c r="B24" s="10" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="D24" s="10"/>
     </row>
     <row r="25" ht="14" spans="1:4">
       <c r="A25" s="10"/>
       <c r="B25" s="10" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="D25" s="10"/>
     </row>
     <row r="26" ht="14" spans="1:4">
       <c r="A26" s="10"/>
       <c r="B26" s="10" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="D26" s="10"/>
     </row>
     <row r="27" ht="14" spans="1:4">
       <c r="A27" s="10"/>
       <c r="B27" s="10" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="D27" s="10"/>
     </row>
     <row r="28" ht="14" spans="1:4">
       <c r="A28" s="10"/>
       <c r="B28" s="10" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="D28" s="10"/>
     </row>
     <row r="29" ht="14" spans="1:4">
       <c r="A29" s="10"/>
       <c r="B29" s="10" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="D29" s="10"/>
     </row>
     <row r="30" ht="14" spans="1:4">
       <c r="A30" s="10"/>
       <c r="B30" s="10" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="D30" s="10"/>
     </row>
     <row r="31" ht="14" spans="1:4">
       <c r="A31" s="10"/>
       <c r="B31" s="10" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="D31" s="10"/>
     </row>
     <row r="32" ht="14" spans="1:4">
       <c r="A32" s="10"/>
       <c r="B32" s="10" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="D32" s="10"/>
     </row>
     <row r="33" ht="14" spans="1:4">
       <c r="A33" s="10"/>
       <c r="B33" s="10" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="D33" s="10"/>
     </row>
     <row r="34" ht="14" spans="1:4">
       <c r="A34" s="10"/>
       <c r="B34" s="10" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
       <c r="D34" s="10"/>
     </row>
     <row r="35" ht="14" spans="1:4">
       <c r="A35" s="10"/>
       <c r="B35" s="10" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="D35" s="10"/>
     </row>
     <row r="36" ht="14" spans="1:4">
       <c r="A36" s="10"/>
       <c r="B36" s="10" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="D36" s="10"/>
     </row>
     <row r="37" ht="14" spans="1:4">
       <c r="A37" s="10"/>
       <c r="B37" s="10" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="D37" s="10"/>
     </row>
     <row r="38" ht="14" spans="1:4">
       <c r="A38" s="10"/>
       <c r="B38" s="10" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="D38" s="10"/>
     </row>
     <row r="39" ht="14" spans="1:4">
       <c r="A39" s="10"/>
       <c r="B39" s="10" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="D39" s="10"/>
     </row>
     <row r="40" ht="14" spans="1:4">
       <c r="A40" s="10"/>
       <c r="B40" s="10" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="D40" s="10"/>
     </row>
     <row r="41" ht="14" spans="1:4">
       <c r="A41" s="10"/>
       <c r="B41" s="10" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="D41" s="10"/>
     </row>
     <row r="42" ht="14" spans="1:4">
       <c r="A42" s="10"/>
       <c r="B42" s="10" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="D42" s="10"/>
     </row>
-    <row r="43" ht="15.5"/>
     <row r="44" ht="14" spans="2:3">
       <c r="B44" s="11" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
     </row>
     <row r="46" ht="14" spans="2:3">
       <c r="B46" s="12" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
spk + synapse + azure
</commit_message>
<xml_diff>
--- a/p/py-25/py-core/topic-list_py.xlsx
+++ b/p/py-25/py-core/topic-list_py.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17600" tabRatio="698" firstSheet="1" activeTab="2"/>
+    <workbookView windowWidth="13830" windowHeight="17600" tabRatio="698"/>
   </bookViews>
   <sheets>
     <sheet name="core" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="503">
   <si>
     <t>Most basic things in py</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>py version</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/python/python-version-history/</t>
   </si>
   <si>
     <t>compare</t>
@@ -1836,10 +1839,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="33">
     <font>
@@ -2381,16 +2384,16 @@
     <xf numFmtId="176" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2956,15 +2959,18 @@
       </c>
       <c r="G3" s="13"/>
     </row>
-    <row r="4" spans="4:7">
+    <row r="4" spans="1:7">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="D4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G4" s="13"/>
     </row>
     <row r="5" spans="4:7">
       <c r="D5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G5" s="13"/>
     </row>
@@ -2973,40 +2979,40 @@
     </row>
     <row r="7" spans="3:3">
       <c r="C7" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="3:3">
       <c r="C9" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="4:4">
       <c r="D10" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="3:3">
       <c r="C12" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="4:4">
       <c r="D13" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:8">
       <c r="A15" s="22" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B15" s="22"/>
       <c r="C15" s="22"/>
@@ -3018,120 +3024,120 @@
     </row>
     <row r="16" spans="3:3">
       <c r="C16" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="3:3">
       <c r="C18" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="4:4">
       <c r="D19" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" spans="4:4">
       <c r="D20" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="4:4">
       <c r="D21" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="4:5">
       <c r="D22" s="9"/>
       <c r="E22" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="3:3">
       <c r="C23" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="4:4">
       <c r="D24" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="3:6">
       <c r="C25" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="3:6">
       <c r="C26" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" spans="3:3">
       <c r="C30" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="31" spans="2:4">
       <c r="B31" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="32" spans="4:4">
       <c r="D32" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B33" s="18"/>
       <c r="C33" s="18"/>
       <c r="D33" s="18" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="18" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="18" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:1">
@@ -3139,33 +3145,33 @@
     </row>
     <row r="37" spans="3:3">
       <c r="C37" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="3:3">
       <c r="C39" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="41" spans="3:3">
       <c r="C41" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="42" spans="4:4">
       <c r="D42" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -3173,53 +3179,53 @@
       <c r="B43" s="19"/>
       <c r="C43" s="19"/>
       <c r="D43" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="4:6">
       <c r="D44" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="45" spans="4:4">
       <c r="D45" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="46" spans="4:4">
       <c r="D46" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="47" spans="4:4">
       <c r="D47" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="48" spans="5:5">
       <c r="E48" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="49" spans="3:3">
       <c r="C49" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="50" spans="4:4">
       <c r="D50" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="53" spans="3:5">
@@ -3298,12 +3304,12 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="2" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="3" spans="1:1">
@@ -3311,7 +3317,7 @@
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="4" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5" spans="1:1">
@@ -3319,32 +3325,32 @@
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="5" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="5" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="6" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="6" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="6" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="5" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="12" spans="1:1">
@@ -3352,7 +3358,7 @@
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="4" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="14" spans="1:1">
@@ -3360,32 +3366,32 @@
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="5" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="5" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="6" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="6" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="6" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="5" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="21" spans="1:1">
@@ -3393,51 +3399,51 @@
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="4" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="3" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="3"/>
       <c r="B24" s="1" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" s="5" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" s="5" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" s="6" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" s="6" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" s="6" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" s="5" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="31" spans="1:1">
@@ -3445,7 +3451,7 @@
     </row>
     <row r="32" spans="1:1">
       <c r="A32" s="4" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="33" spans="1:1">
@@ -3453,32 +3459,32 @@
     </row>
     <row r="34" spans="1:1">
       <c r="A34" s="5" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" s="5" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" s="6" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" s="6" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" s="6" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" s="5" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="40" spans="1:1">
@@ -3486,7 +3492,7 @@
     </row>
     <row r="41" spans="1:1">
       <c r="A41" s="4" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
     <row r="42" spans="1:1">
@@ -3494,32 +3500,32 @@
     </row>
     <row r="43" spans="1:1">
       <c r="A43" s="5" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" s="5" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" s="6" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" s="6" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" s="6" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" s="5" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="49" spans="1:1">
@@ -3527,7 +3533,7 @@
     </row>
     <row r="50" spans="1:1">
       <c r="A50" s="4" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="51" spans="1:1">
@@ -3535,32 +3541,32 @@
     </row>
     <row r="52" spans="1:1">
       <c r="A52" s="5" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="53" spans="1:1">
       <c r="A53" s="5" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" s="6" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="55" spans="1:1">
       <c r="A55" s="6" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="56" spans="1:1">
       <c r="A56" s="6" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="57" spans="1:1">
       <c r="A57" s="5" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="58" spans="1:1">
@@ -3568,7 +3574,7 @@
     </row>
     <row r="59" spans="1:1">
       <c r="A59" s="4" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="60" spans="1:1">
@@ -3576,32 +3582,32 @@
     </row>
     <row r="61" spans="1:1">
       <c r="A61" s="5" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="62" spans="1:1">
       <c r="A62" s="5" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="63" spans="1:1">
       <c r="A63" s="6" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="64" spans="1:1">
       <c r="A64" s="6" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="65" spans="1:1">
       <c r="A65" s="6" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="66" spans="1:1">
       <c r="A66" s="5" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="67" spans="1:1">
@@ -3609,37 +3615,37 @@
     </row>
     <row r="68" spans="1:1">
       <c r="A68" s="4" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="69" spans="1:1">
       <c r="A69" s="2" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="70" spans="1:1">
       <c r="A70" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="71" spans="1:1">
       <c r="A71" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="73" spans="1:1">
       <c r="A73" s="7" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="74" spans="1:1">
       <c r="A74" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="75" spans="1:1">
       <c r="A75" s="1" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
   </sheetData>
@@ -3666,7 +3672,7 @@
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3691,32 +3697,32 @@
     </row>
     <row r="3" spans="3:3">
       <c r="C3" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="4:4">
       <c r="D4" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="3:3">
       <c r="C6" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="3:3">
       <c r="C7" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="3:3">
       <c r="C9" s="20" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="3:5">
       <c r="C11" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
@@ -3724,87 +3730,87 @@
     <row r="12" spans="3:5">
       <c r="C12" s="9"/>
       <c r="D12" s="21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E12" s="9"/>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E13" s="9"/>
     </row>
     <row r="14" spans="3:5">
       <c r="C14" s="9"/>
       <c r="D14" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E14" s="9"/>
     </row>
     <row r="15" spans="3:5">
       <c r="C15" s="9"/>
       <c r="D15" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E15" s="9"/>
     </row>
     <row r="16" spans="3:5">
       <c r="C16" s="9"/>
       <c r="D16" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E16" s="9"/>
     </row>
     <row r="17" spans="3:5">
       <c r="C17" s="9"/>
       <c r="D17" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E17" s="9"/>
     </row>
     <row r="18" spans="3:5">
       <c r="C18" s="9"/>
       <c r="D18" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E18" s="9"/>
     </row>
     <row r="19" spans="3:5">
       <c r="C19" s="9"/>
       <c r="D19" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E19" s="9"/>
     </row>
     <row r="20" spans="3:5">
       <c r="C20" s="9"/>
       <c r="D20" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E20" s="9"/>
     </row>
     <row r="21" spans="3:5">
       <c r="C21" s="9"/>
       <c r="D21" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E21" s="9"/>
     </row>
     <row r="22" spans="3:5">
       <c r="C22" s="9"/>
       <c r="D22" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E22" s="9"/>
     </row>
     <row r="23" spans="3:5">
       <c r="C23" s="9"/>
       <c r="D23" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E23" s="9"/>
     </row>
@@ -3815,17 +3821,17 @@
     </row>
     <row r="25" spans="3:3">
       <c r="C25" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="3:3">
       <c r="C26" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" ht="27" customHeight="1" spans="1:8">
       <c r="A27" s="22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B27" s="22"/>
       <c r="C27" s="22"/>
@@ -3839,7 +3845,7 @@
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="23" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D28" s="22"/>
       <c r="E28" s="22"/>
@@ -3849,7 +3855,7 @@
     </row>
     <row r="29" ht="16" customHeight="1" spans="1:8">
       <c r="A29" s="24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C29" s="23"/>
       <c r="D29" s="22"/>
@@ -3860,7 +3866,7 @@
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:8">
       <c r="A30" s="23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B30" s="22"/>
       <c r="C30" s="23"/>
@@ -3872,10 +3878,10 @@
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:8">
       <c r="A31" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B31" s="24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C31" s="23"/>
       <c r="D31" s="22"/>
@@ -3886,7 +3892,7 @@
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:8">
       <c r="A32" s="23" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B32" s="22"/>
       <c r="C32" s="23"/>
@@ -3908,11 +3914,11 @@
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:8">
       <c r="A34" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
@@ -3923,7 +3929,7 @@
     <row r="35" ht="16" customHeight="1" spans="1:8">
       <c r="A35" s="9"/>
       <c r="B35" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
@@ -3934,10 +3940,10 @@
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:8">
       <c r="A36" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
@@ -3948,14 +3954,14 @@
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:8">
       <c r="A37" s="23" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C37" s="9"/>
       <c r="D37" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E37" s="9"/>
       <c r="F37" s="23"/>
@@ -3965,11 +3971,11 @@
     <row r="38" ht="16" customHeight="1" spans="1:8">
       <c r="A38" s="9"/>
       <c r="B38" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E38" s="9"/>
       <c r="F38" s="23"/>
@@ -3981,11 +3987,11 @@
       <c r="B39" s="23"/>
       <c r="C39" s="23"/>
       <c r="D39" s="23" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E39" s="23"/>
       <c r="F39" s="23" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G39" s="23"/>
       <c r="H39" s="22"/>
@@ -3994,7 +4000,7 @@
       <c r="A40" s="23"/>
       <c r="B40" s="23"/>
       <c r="C40" s="23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D40" s="23"/>
       <c r="E40" s="23"/>
@@ -4006,7 +4012,7 @@
       <c r="A41" s="23"/>
       <c r="B41" s="23"/>
       <c r="C41" s="23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D41" s="23"/>
       <c r="E41" s="23"/>
@@ -4016,13 +4022,13 @@
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:8">
       <c r="A42" s="23" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D42" s="23"/>
       <c r="E42" s="23"/>
@@ -4033,7 +4039,7 @@
     <row r="43" ht="16" customHeight="1" spans="1:8">
       <c r="A43" s="23"/>
       <c r="B43" s="23" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C43" s="23"/>
       <c r="D43" s="23"/>
@@ -4045,7 +4051,7 @@
     <row r="44" ht="16" customHeight="1" spans="1:8">
       <c r="A44" s="23"/>
       <c r="B44" s="23" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C44" s="23"/>
       <c r="D44" s="23"/>
@@ -4068,7 +4074,7 @@
       <c r="A46" s="23"/>
       <c r="B46" s="23"/>
       <c r="C46" s="23" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D46" s="23"/>
       <c r="E46" s="23"/>
@@ -4079,11 +4085,11 @@
     <row r="47" ht="16" customHeight="1" spans="1:8">
       <c r="A47" s="23"/>
       <c r="B47" s="23" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C47" s="23"/>
       <c r="D47" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E47" s="23"/>
       <c r="F47" s="23"/>
@@ -4092,11 +4098,11 @@
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:8">
       <c r="A48" s="23" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B48" s="23"/>
       <c r="C48" s="23" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D48" s="23"/>
       <c r="E48" s="23"/>
@@ -4308,7 +4314,7 @@
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D69" s="9"/>
       <c r="E69" s="3"/>
@@ -4319,7 +4325,7 @@
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D70" s="9"/>
       <c r="E70" s="3"/>
@@ -4331,7 +4337,7 @@
       <c r="B71" s="3"/>
       <c r="C71" s="9"/>
       <c r="D71" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
@@ -4343,16 +4349,16 @@
     </row>
     <row r="73" spans="1:3">
       <c r="A73" s="25" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B73" s="9"/>
       <c r="C73" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="74" spans="1:1">
       <c r="A74" s="26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -4385,7 +4391,7 @@
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -4410,100 +4416,100 @@
     </row>
     <row r="3" spans="2:7">
       <c r="B3" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G3" s="13"/>
     </row>
     <row r="4" spans="3:7">
       <c r="C4" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G4" s="13"/>
     </row>
     <row r="5" spans="4:7">
       <c r="D5" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G5" s="13"/>
     </row>
     <row r="6" spans="4:7">
       <c r="D6" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G6" s="13"/>
     </row>
     <row r="7" spans="3:3">
       <c r="C7" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="4:4">
       <c r="D8" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="5:5">
       <c r="E9" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="4:4">
       <c r="D10" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="4:4">
       <c r="D11" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="5:5">
       <c r="E12" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="3:3">
       <c r="C14" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="15" spans="4:4">
       <c r="D15" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16" ht="14.5" spans="2:4">
       <c r="B16" s="17" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" ht="14.5" spans="2:5">
       <c r="B17" s="17"/>
       <c r="C17" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" ht="14.5" spans="2:4">
       <c r="B18" s="17"/>
       <c r="D18" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="19" ht="14.5" spans="2:2">
@@ -4511,11 +4517,11 @@
     </row>
     <row r="20" ht="14.5" spans="1:3">
       <c r="A20" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="21" ht="14.5" spans="2:2">
@@ -4524,21 +4530,21 @@
     <row r="22" ht="14.5" spans="2:3">
       <c r="B22" s="17"/>
       <c r="C22" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23" ht="14.5" spans="2:4">
       <c r="B23" s="17" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="24" ht="14.5" spans="2:3">
       <c r="B24" s="17"/>
       <c r="C24" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="25" ht="14.5" spans="2:2">
@@ -4546,317 +4552,317 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="27" spans="3:5">
       <c r="C27" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" spans="2:4">
       <c r="B29" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30" spans="4:4">
       <c r="D30" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" spans="4:4">
       <c r="D31" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="32" spans="2:4">
       <c r="B32" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="34" spans="3:3">
       <c r="C34" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="35" spans="3:3">
       <c r="C35" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="36" spans="4:4">
       <c r="D36" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="37" spans="2:5">
       <c r="B37" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="38" spans="2:6">
       <c r="B38" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="40" spans="2:4">
       <c r="B40" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="42" spans="2:2">
       <c r="B42" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="44" spans="2:2">
       <c r="B44" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="45" spans="4:4">
       <c r="D45" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="46" spans="5:5">
       <c r="E46" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="48" spans="2:4">
       <c r="B48" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="49" spans="4:4">
       <c r="D49" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="50" spans="3:3">
       <c r="C50" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="51" spans="4:4">
       <c r="D51" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="53" spans="5:5">
       <c r="E53" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="55" spans="4:4">
       <c r="D55" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="56" spans="4:4">
       <c r="D56" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="59" spans="2:2">
       <c r="B59" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="61" spans="2:2">
       <c r="B61" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="62" spans="3:3">
       <c r="C62" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="63" spans="4:4">
       <c r="D63" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="64" spans="4:4">
       <c r="D64" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="65" spans="4:4">
       <c r="D65" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="67" spans="3:3">
       <c r="C67" s="9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="68" spans="3:4">
       <c r="C68" s="9"/>
       <c r="D68" s="9" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="69" spans="3:5">
       <c r="C69" s="9"/>
       <c r="E69" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="70" spans="3:4">
       <c r="C70" s="9"/>
       <c r="D70" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="71" spans="3:5">
       <c r="C71" s="9"/>
       <c r="E71" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="72" spans="3:4">
       <c r="C72" s="9"/>
       <c r="D72" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="73" spans="3:3">
@@ -5009,29 +5015,29 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="2:4">
       <c r="B4" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5" spans="2:5">
       <c r="B5" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -5060,7 +5066,7 @@
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -5085,106 +5091,106 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="2:2">
       <c r="B4" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="2:2">
       <c r="B5" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="9" spans="4:4">
       <c r="D9" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="4:4">
       <c r="D11" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12" spans="5:5">
       <c r="E12" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="13" spans="3:3">
       <c r="C13" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14" spans="2:4">
       <c r="B14" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="4:4">
       <c r="D16" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
@@ -5195,19 +5201,19 @@
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
@@ -5218,33 +5224,33 @@
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="9" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F23" s="9"/>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F24" s="9"/>
     </row>
@@ -5253,29 +5259,29 @@
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="9" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
@@ -5284,10 +5290,10 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="9" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
@@ -5338,23 +5344,23 @@
     </row>
     <row r="34" spans="1:9">
       <c r="A34" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H34" s="10"/>
       <c r="I34" s="10"/>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G36" s="16">
         <v>5</v>
@@ -5362,42 +5368,42 @@
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="39" spans="5:5">
       <c r="E39" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="41" spans="2:2">
       <c r="B41" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>
@@ -5425,7 +5431,7 @@
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" s="11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -5447,7 +5453,7 @@
     </row>
     <row r="3" spans="3:5">
       <c r="C3" s="10" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
@@ -5455,66 +5461,66 @@
     <row r="4" spans="3:5">
       <c r="C4" s="10"/>
       <c r="D4" s="10" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="3:5">
       <c r="C5" s="10"/>
       <c r="D5" s="11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E5" s="10"/>
     </row>
     <row r="6" spans="3:5">
       <c r="C6" s="10"/>
       <c r="D6" s="11" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E6" s="10"/>
     </row>
     <row r="7" spans="3:5">
       <c r="C7" s="10"/>
       <c r="D7" s="11" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E7" s="10"/>
     </row>
     <row r="8" spans="3:5">
       <c r="C8" s="10"/>
       <c r="D8" s="10" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E8" s="10"/>
     </row>
     <row r="9" spans="4:4">
       <c r="D9" s="11" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="10" spans="4:4">
       <c r="D10" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" spans="4:4">
       <c r="D11" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="12" spans="4:4">
       <c r="D12" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="13" spans="4:4">
       <c r="D13" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="14" spans="4:4">
       <c r="D14" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="15" spans="4:4">
@@ -5531,150 +5537,150 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="20" spans="2:3">
       <c r="B20" s="11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="11" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="11" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23" spans="4:4">
       <c r="D23" s="11" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="24" spans="4:4">
       <c r="D24" s="11" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="25" spans="4:4">
       <c r="D25" s="11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="11" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="28" spans="5:5">
       <c r="E28" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="29" spans="4:4">
       <c r="D29" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="31" spans="3:3">
       <c r="C31" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="33" spans="4:5">
       <c r="D33" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="35" spans="3:4">
       <c r="C35" s="10" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D35" s="10"/>
     </row>
     <row r="36" spans="3:4">
       <c r="C36" s="10"/>
       <c r="D36" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="37" spans="3:4">
       <c r="C37" s="10"/>
       <c r="D37" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="38" spans="3:4">
       <c r="C38" s="10" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D38" s="10"/>
     </row>
@@ -5684,314 +5690,314 @@
     </row>
     <row r="40" spans="3:4">
       <c r="C40" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D40" s="10"/>
     </row>
     <row r="41" spans="3:4">
       <c r="C41" s="10"/>
       <c r="D41" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="43" spans="3:3">
       <c r="C43" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="44" spans="4:5">
       <c r="D44" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="45" spans="5:5">
       <c r="E45" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="47" spans="4:4">
       <c r="D47" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="48" spans="5:5">
       <c r="E48" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="49" spans="5:5">
       <c r="E49" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="50" spans="5:5">
       <c r="E50" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="52" spans="3:3">
       <c r="C52" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="53" spans="4:5">
       <c r="D53" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="54" spans="5:5">
       <c r="E54" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="55" spans="4:4">
       <c r="D55" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="57" spans="2:4">
       <c r="B57" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="59" spans="3:3">
       <c r="C59" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="60" spans="4:4">
       <c r="D60" s="11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="61" spans="3:3">
       <c r="C61" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="62" spans="2:4">
       <c r="B62" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D62" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="63" spans="2:2">
       <c r="B63" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="64" spans="3:3">
       <c r="C64" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="65" spans="4:5">
       <c r="D65" s="11" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D67" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="68" spans="2:2">
       <c r="B68" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="69" spans="2:2">
       <c r="B69" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="71" spans="3:3">
       <c r="C71" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="72" spans="4:4">
       <c r="D72" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="73" spans="4:4">
       <c r="D73" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="74" spans="4:4">
       <c r="D74" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="75" spans="4:4">
       <c r="D75" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="77" spans="2:4">
       <c r="B77" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D77" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C78" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="79" spans="4:4">
       <c r="D79" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="80" spans="2:3">
       <c r="B80" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="81" spans="3:3">
       <c r="C81" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C82" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="83" spans="4:4">
       <c r="D83" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="84" spans="4:4">
       <c r="D84" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C85" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="86" spans="3:3">
       <c r="C86" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="87" spans="4:4">
       <c r="D87" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="88" spans="4:4">
       <c r="D88" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C91" s="11" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="92" spans="4:4">
       <c r="D92" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="93" spans="4:4">
       <c r="D93" s="11" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="94" spans="1:7">
       <c r="A94" s="11" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C94" s="11" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G94" s="14">
         <v>5</v>
@@ -6042,39 +6048,39 @@
     </row>
     <row r="3" spans="3:5">
       <c r="C3" s="1" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="4" spans="3:5">
       <c r="C4" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="5" spans="3:5">
       <c r="C5" s="1" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="6" spans="3:3">
       <c r="C6" s="1" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="7" spans="3:5">
       <c r="C7" s="1" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
   </sheetData>
@@ -6112,37 +6118,37 @@
   <sheetData>
     <row r="3" spans="3:3">
       <c r="C3" s="8" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="5" spans="3:3">
       <c r="C5" s="8" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="7" spans="3:3">
       <c r="C7" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="8" ht="14" spans="4:4">
       <c r="D8" s="9" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="9" spans="3:3">
       <c r="C9" s="8" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="11" spans="3:3">
       <c r="C11" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="13" ht="14" spans="1:4">
       <c r="A13" s="10" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -6150,7 +6156,7 @@
     </row>
     <row r="14" ht="14" spans="1:4">
       <c r="A14" s="10" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -6159,50 +6165,50 @@
     <row r="15" ht="14" spans="1:4">
       <c r="A15" s="10"/>
       <c r="B15" s="10" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D15" s="10"/>
     </row>
     <row r="16" ht="14" spans="1:4">
       <c r="A16" s="10"/>
       <c r="B16" s="10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D16" s="10"/>
     </row>
     <row r="17" ht="14" spans="1:4">
       <c r="A17" s="10"/>
       <c r="B17" s="10" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D17" s="10"/>
     </row>
     <row r="18" ht="14" spans="1:4">
       <c r="A18" s="10"/>
       <c r="B18" s="10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D18" s="10"/>
     </row>
     <row r="19" ht="14" spans="1:4">
       <c r="A19" s="10"/>
       <c r="B19" s="10" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D19" s="10"/>
     </row>
@@ -6210,244 +6216,244 @@
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D20" s="10"/>
     </row>
     <row r="21" ht="14" spans="1:4">
       <c r="A21" s="10"/>
       <c r="B21" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D21" s="10"/>
     </row>
     <row r="22" ht="14" spans="1:4">
       <c r="A22" s="10"/>
       <c r="B22" s="10" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D22" s="10"/>
     </row>
     <row r="23" ht="14" spans="1:4">
       <c r="A23" s="10"/>
       <c r="B23" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D23" s="10"/>
     </row>
     <row r="24" ht="14" spans="1:4">
       <c r="A24" s="10"/>
       <c r="B24" s="10" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D24" s="10"/>
     </row>
     <row r="25" ht="14" spans="1:4">
       <c r="A25" s="10"/>
       <c r="B25" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="C25" s="10" t="s">
         <v>413</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>412</v>
       </c>
       <c r="D25" s="10"/>
     </row>
     <row r="26" ht="14" spans="1:4">
       <c r="A26" s="10"/>
       <c r="B26" s="10" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D26" s="10"/>
     </row>
     <row r="27" ht="14" spans="1:4">
       <c r="A27" s="10"/>
       <c r="B27" s="10" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D27" s="10"/>
     </row>
     <row r="28" ht="14" spans="1:4">
       <c r="A28" s="10"/>
       <c r="B28" s="10" t="s">
+        <v>417</v>
+      </c>
+      <c r="C28" s="10" t="s">
         <v>416</v>
-      </c>
-      <c r="C28" s="10" t="s">
-        <v>415</v>
       </c>
       <c r="D28" s="10"/>
     </row>
     <row r="29" ht="14" spans="1:4">
       <c r="A29" s="10"/>
       <c r="B29" s="10" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D29" s="10"/>
     </row>
     <row r="30" ht="14" spans="1:4">
       <c r="A30" s="10"/>
       <c r="B30" s="10" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D30" s="10"/>
     </row>
     <row r="31" ht="14" spans="1:4">
       <c r="A31" s="10"/>
       <c r="B31" s="10" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D31" s="10"/>
     </row>
     <row r="32" ht="14" spans="1:4">
       <c r="A32" s="10"/>
       <c r="B32" s="10" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D32" s="10"/>
     </row>
     <row r="33" ht="14" spans="1:4">
       <c r="A33" s="10"/>
       <c r="B33" s="10" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D33" s="10"/>
     </row>
     <row r="34" ht="14" spans="1:4">
       <c r="A34" s="10"/>
       <c r="B34" s="10" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D34" s="10"/>
     </row>
     <row r="35" ht="14" spans="1:4">
       <c r="A35" s="10"/>
       <c r="B35" s="10" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D35" s="10"/>
     </row>
     <row r="36" ht="14" spans="1:4">
       <c r="A36" s="10"/>
       <c r="B36" s="10" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D36" s="10"/>
     </row>
     <row r="37" ht="14" spans="1:4">
       <c r="A37" s="10"/>
       <c r="B37" s="10" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D37" s="10"/>
     </row>
     <row r="38" ht="14" spans="1:4">
       <c r="A38" s="10"/>
       <c r="B38" s="10" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D38" s="10"/>
     </row>
     <row r="39" ht="14" spans="1:4">
       <c r="A39" s="10"/>
       <c r="B39" s="10" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D39" s="10"/>
     </row>
     <row r="40" ht="14" spans="1:4">
       <c r="A40" s="10"/>
       <c r="B40" s="10" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D40" s="10"/>
     </row>
     <row r="41" ht="14" spans="1:4">
       <c r="A41" s="10"/>
       <c r="B41" s="10" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D41" s="10"/>
     </row>
     <row r="42" ht="14" spans="1:4">
       <c r="A42" s="10"/>
       <c r="B42" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D42" s="10"/>
     </row>
     <row r="44" ht="14" spans="2:3">
       <c r="B44" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="46" ht="14" spans="2:3">
       <c r="B46" s="12" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
   </sheetData>

</xml_diff>